<commit_message>
feat(tg-cotizador): quitar columna 'Piezas por unidad de cobro' (rinde solo por geometria)
El rinde efectivo ya se calculaba por geometria desde que el catalogo v4
es la fuente; la columna estaba vacia en las 3 versiones y solo invitaba a
cargar a mano un dato que el sistema deriva. Se elimina la columna G de
Productos (corriendo Sinonimos/Formato una posicion a la izquierda) y se
limpian las referencias: chunk.ts ya no la lee, el parametro rinde_cargado
de cotizar() queda muerto y se borra, y la hoja Instrucciones +
instrucciones-cliente.md dejan de mencionarla.

Verificado: 131/131 casos, 11 rindes, 116 chunks identicos al antes (la
columna vacia no aportaba nada), validar-catalogo sin errores.

Nota: listar-casos.mjs y cargar-casos-cobertura.mjs NO se tocan — su
columna 'Piezas por unidad de cobro' es la F de Casos de prueba, que se
conserva (es el unico chequeo de rinde del gate).
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v4.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v4.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="1058">
   <si>
     <t xml:space="preserve">CÓMO CARGAR PRODUCTOS NUEVOS</t>
   </si>
@@ -3184,6 +3184,21 @@
   </si>
   <si>
     <t xml:space="preserve">Los cambios NO llegan al bot hasta que se ingesta desde ahí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE DÓNDE SALE EL RINDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya NO se carga a mano: el rinde sale SIEMPRE de la geometría. La geometría se declara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNA vez por material en la hoja Materiales ('Área útil ancho/alto (cm)' y 'Separación (cm)')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y el rinde se calcula solo, con la fórmula de la PARTE 1: el visor lo calcula para las</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medidas de referencia y el bot para cualquier otra medida que pida el cliente.</t>
   </si>
 </sst>
 </file>
@@ -3619,7 +3634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A163"/>
+  <dimension ref="A1:A150"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="105" customWidth="1" style="28" min="1" max="1"/>
@@ -3640,30 +3655,30 @@
         <v>983</v>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="16" t="s">
+    <row r="4">
+      <c r="A4" s="16" t="s">
         <v>984</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="16" t="s">
         <v>985</v>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="16" t="s">
+    <row r="7">
+      <c r="A7" s="16" t="s">
         <v>986</v>
       </c>
     </row>
-    <row r="9"/>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="16" t="s">
+        <v>987</v>
+      </c>
+    </row>
     <row r="10"/>
-    <row r="11">
-      <c r="A11" s="16" t="s">
-        <v>987</v>
-      </c>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="16" t="s">
         <v>988</v>
@@ -3694,12 +3709,12 @@
         <v>993</v>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="16" t="s">
+    <row r="18">
+      <c r="A18" s="16" t="s">
         <v>994</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="16" t="s">
         <v>995</v>
@@ -3720,29 +3735,29 @@
         <v>998</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="16" t="s">
+    <row r="24">
+      <c r="A24" s="16" t="s">
         <v>999</v>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="16" t="s">
         <v>1000</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="16" t="s">
+    <row r="27">
+      <c r="A27" s="16" t="s">
         <v>1001</v>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="16" t="s">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="16" t="s">
         <v>1002</v>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="16" t="s">
         <v>1003</v>
@@ -3763,12 +3778,12 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="16" t="s">
+    <row r="35">
+      <c r="A35" s="16" t="s">
         <v>1007</v>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="16" t="s">
         <v>1008</v>
@@ -3779,12 +3794,12 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="16" t="s">
+    <row r="39">
+      <c r="A39" s="16" t="s">
         <v>1010</v>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="16" t="s">
         <v>1011</v>
@@ -3795,12 +3810,12 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44">
-      <c r="A44" s="16" t="s">
+    <row r="43">
+      <c r="A43" s="16" t="s">
         <v>1013</v>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="16" t="s">
         <v>1014</v>
@@ -3811,22 +3826,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47"/>
+    <row r="47">
+      <c r="A47" s="16" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="48"/>
     <row r="49"/>
     <row r="50"/>
     <row r="51"/>
-    <row r="52">
-      <c r="A52" s="16" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="53"/>
-    <row r="54">
-      <c r="A54" s="16" t="s">
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="16" t="s">
         <v>7</v>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="16" t="s">
         <v>8</v>
@@ -3857,12 +3872,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61"/>
-    <row r="62">
-      <c r="A62" s="16" t="s">
+    <row r="61">
+      <c r="A61" s="16" t="s">
         <v>1018</v>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="16" t="s">
         <v>16</v>
@@ -3873,23 +3888,23 @@
         <v>17</v>
       </c>
     </row>
-    <row r="65"/>
-    <row r="66">
-      <c r="A66" s="16" t="s">
+    <row r="65">
+      <c r="A65" s="16" t="s">
         <v>18</v>
       </c>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="68"/>
-    <row r="69">
-      <c r="A69" s="16" t="s">
+    <row r="68">
+      <c r="A68" s="16" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="69"/>
     <row r="70">
       <c r="A70" s="16" t="s">
         <v>21</v>
@@ -3910,12 +3925,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="74"/>
-    <row r="75">
-      <c r="A75" s="16" t="s">
+    <row r="74">
+      <c r="A74" s="16" t="s">
         <v>25</v>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="16" t="s">
         <v>1019</v>
@@ -3936,12 +3951,12 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="80"/>
-    <row r="81">
-      <c r="A81" s="16" t="s">
+    <row r="80">
+      <c r="A80" s="16" t="s">
         <v>1023</v>
       </c>
     </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" s="16" t="s">
         <v>1024</v>
@@ -3957,12 +3972,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="85"/>
-    <row r="86">
-      <c r="A86" s="16" t="s">
+    <row r="85">
+      <c r="A85" s="16" t="s">
         <v>28</v>
       </c>
     </row>
+    <row r="86"/>
     <row r="87">
       <c r="A87" s="16" t="s">
         <v>1026</v>
@@ -3978,12 +3993,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="90"/>
-    <row r="91">
-      <c r="A91" s="16" t="s">
+    <row r="90">
+      <c r="A90" s="16" t="s">
         <v>32</v>
       </c>
     </row>
+    <row r="91"/>
     <row r="92">
       <c r="A92" s="16" t="s">
         <v>33</v>
@@ -3991,281 +4006,259 @@
     </row>
     <row r="93">
       <c r="A93" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="98"/>
     <row r="99">
       <c r="A99" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="16" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="16" t="s">
-        <v>42</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="104"/>
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="s">
+        <v>1055</v>
+      </c>
+    </row>
     <row r="105">
       <c r="A105" s="16" t="s">
-        <v>49</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="16" t="s">
-        <v>50</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="16" t="s">
-        <v>1027</v>
+        <v>52</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="16" t="s">
-        <v>1028</v>
+        <v>53</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="16" t="s">
-        <v>52</v>
+        <v>98</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="16" t="s">
-        <v>53</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="16" t="s">
-        <v>55</v>
-      </c>
-    </row>
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="16" t="s">
-        <v>1029</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="16" t="s">
-        <v>98</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="16" t="s">
-        <v>1030</v>
-      </c>
-    </row>
-    <row r="116"/>
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="16" t="s">
+        <v>1035</v>
+      </c>
+    </row>
     <row r="117">
       <c r="A117" s="16" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="16" t="s">
-        <v>1032</v>
-      </c>
-    </row>
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="16" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="16" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="16" t="s">
-        <v>1035</v>
-      </c>
-    </row>
-    <row r="122"/>
-    <row r="123">
-      <c r="A123" s="16" t="s">
-        <v>1036</v>
-      </c>
-    </row>
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="16" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="16" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="16" t="s">
-        <v>1038</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="16" t="s">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="127"/>
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="126"/>
+    <row r="127">
+      <c r="A127" s="16" t="s">
+        <v>1043</v>
+      </c>
+    </row>
     <row r="128">
       <c r="A128" s="16" t="s">
-        <v>1040</v>
+        <v>57</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="16" t="s">
-        <v>1041</v>
-      </c>
-    </row>
-    <row r="130"/>
-    <row r="131">
-      <c r="A131" s="16" t="s">
-        <v>1042</v>
-      </c>
-    </row>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="131"/>
     <row r="132">
       <c r="A132" s="16" t="s">
-        <v>1043</v>
+        <v>60</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="16" t="s">
-        <v>57</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="16" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="135"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="s">
+        <v>63</v>
+      </c>
+    </row>
     <row r="136">
       <c r="A136" s="16" t="s">
-        <v>59</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="16" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="16" t="s">
-        <v>1044</v>
-      </c>
-    </row>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="138"/>
     <row r="139">
       <c r="A139" s="16" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="16" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="16" t="s">
-        <v>1045</v>
-      </c>
-    </row>
-    <row r="142"/>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="141"/>
+    <row r="142">
+      <c r="A142" s="16" t="s">
+        <v>1046</v>
+      </c>
+    </row>
     <row r="143">
       <c r="A143" s="16" t="s">
-        <v>84</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="16" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="145"/>
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="16" t="s">
+        <v>1049</v>
+      </c>
+    </row>
     <row r="146">
       <c r="A146" s="16" t="s">
-        <v>86</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="16" t="s">
-        <v>1046</v>
+        <v>90</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="16" t="s">
-        <v>1047</v>
+        <v>117</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="16" t="s">
-        <v>1048</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="16" t="s">
-        <v>1049</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="16" t="s">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="16" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="16" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="16" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="155"/>
-    <row r="156">
-      <c r="A156" s="16" t="s">
         <v>1052</v>
       </c>
     </row>
@@ -4461,7 +4454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I167"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="21" customWidth="1" style="28" min="1" max="1"/>
@@ -4493,12 +4486,9 @@
         <v>160</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="I1" s="20" t="s">
         <v>163</v>
       </c>
     </row>
@@ -5141,7 +5131,7 @@
       <c r="F33" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="H33" s="28" t="s">
+      <c r="G33" s="28" t="s">
         <v>217</v>
       </c>
     </row>
@@ -5204,7 +5194,7 @@
       <c r="F36" s="32" t="n">
         <v>70</v>
       </c>
-      <c r="H36" s="28" t="s">
+      <c r="G36" s="28" t="s">
         <v>227</v>
       </c>
     </row>
@@ -5227,7 +5217,7 @@
       <c r="F37" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="H37" s="28" t="s">
+      <c r="G37" s="28" t="s">
         <v>230</v>
       </c>
     </row>
@@ -5504,10 +5494,10 @@
       <c r="D51" s="25" t="s">
         <v>272</v>
       </c>
+      <c r="G51" s="28" t="s">
+        <v>273</v>
+      </c>
       <c r="H51" s="28" t="s">
-        <v>273</v>
-      </c>
-      <c r="I51" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5530,7 +5520,7 @@
       <c r="F52" s="32" t="n">
         <v>11</v>
       </c>
-      <c r="H52" s="28" t="s">
+      <c r="G52" s="28" t="s">
         <v>278</v>
       </c>
     </row>
@@ -5547,10 +5537,10 @@
       <c r="D53" s="25" t="s">
         <v>281</v>
       </c>
+      <c r="G53" s="28" t="s">
+        <v>282</v>
+      </c>
       <c r="H53" s="28" t="s">
-        <v>282</v>
-      </c>
-      <c r="I53" s="28" t="s">
         <v>283</v>
       </c>
     </row>
@@ -5573,7 +5563,7 @@
       <c r="F54" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="H54" s="28" t="s">
+      <c r="G54" s="28" t="s">
         <v>286</v>
       </c>
     </row>
@@ -5590,10 +5580,10 @@
       <c r="D55" s="25" t="s">
         <v>289</v>
       </c>
+      <c r="G55" s="28" t="s">
+        <v>290</v>
+      </c>
       <c r="H55" s="28" t="s">
-        <v>290</v>
-      </c>
-      <c r="I55" s="28" t="s">
         <v>291</v>
       </c>
     </row>
@@ -5610,7 +5600,7 @@
       <c r="D56" s="25" t="s">
         <v>292</v>
       </c>
-      <c r="I56" s="28" t="s">
+      <c r="H56" s="28" t="s">
         <v>291</v>
       </c>
     </row>
@@ -5627,10 +5617,10 @@
       <c r="D57" s="25" t="s">
         <v>294</v>
       </c>
+      <c r="G57" s="28" t="s">
+        <v>296</v>
+      </c>
       <c r="H57" s="28" t="s">
-        <v>296</v>
-      </c>
-      <c r="I57" s="28" t="s">
         <v>297</v>
       </c>
     </row>
@@ -5647,7 +5637,7 @@
       <c r="D58" s="25" t="s">
         <v>298</v>
       </c>
-      <c r="I58" s="28" t="s">
+      <c r="H58" s="28" t="s">
         <v>297</v>
       </c>
     </row>
@@ -5664,10 +5654,10 @@
       <c r="D59" s="25" t="s">
         <v>302</v>
       </c>
+      <c r="G59" s="28" t="s">
+        <v>303</v>
+      </c>
       <c r="H59" s="28" t="s">
-        <v>303</v>
-      </c>
-      <c r="I59" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5684,7 +5674,7 @@
       <c r="D60" s="25" t="s">
         <v>304</v>
       </c>
-      <c r="I60" s="28" t="s">
+      <c r="H60" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5701,10 +5691,10 @@
       <c r="D61" s="25" t="s">
         <v>308</v>
       </c>
+      <c r="G61" s="28" t="s">
+        <v>309</v>
+      </c>
       <c r="H61" s="28" t="s">
-        <v>309</v>
-      </c>
-      <c r="I61" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5721,7 +5711,7 @@
       <c r="D62" s="25" t="s">
         <v>310</v>
       </c>
-      <c r="I62" s="28" t="s">
+      <c r="H62" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5738,7 +5728,7 @@
       <c r="D63" s="25" t="s">
         <v>312</v>
       </c>
-      <c r="I63" s="28" t="s">
+      <c r="H63" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -5755,7 +5745,7 @@
       <c r="D64" s="25" t="s">
         <v>315</v>
       </c>
-      <c r="I64" s="28" t="s">
+      <c r="H64" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -5772,7 +5762,7 @@
       <c r="D65" s="25" t="s">
         <v>317</v>
       </c>
-      <c r="I65" s="28" t="s">
+      <c r="H65" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5789,7 +5779,7 @@
       <c r="D66" s="25" t="s">
         <v>319</v>
       </c>
-      <c r="I66" s="28" t="s">
+      <c r="H66" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5806,10 +5796,10 @@
       <c r="D67" s="25" t="s">
         <v>321</v>
       </c>
+      <c r="G67" s="28" t="s">
+        <v>323</v>
+      </c>
       <c r="H67" s="28" t="s">
-        <v>323</v>
-      </c>
-      <c r="I67" s="28" t="s">
         <v>324</v>
       </c>
     </row>
@@ -5826,10 +5816,10 @@
       <c r="D68" s="25" t="s">
         <v>325</v>
       </c>
+      <c r="G68" s="28" t="s">
+        <v>327</v>
+      </c>
       <c r="H68" s="28" t="s">
-        <v>327</v>
-      </c>
-      <c r="I68" s="28" t="s">
         <v>328</v>
       </c>
     </row>
@@ -5846,10 +5836,10 @@
       <c r="D69" s="25" t="s">
         <v>331</v>
       </c>
-      <c r="H69" t="s">
+      <c r="G69" t="s">
         <v>332</v>
       </c>
-      <c r="I69" s="28" t="s">
+      <c r="H69" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5866,10 +5856,10 @@
       <c r="D70" s="25" t="s">
         <v>333</v>
       </c>
+      <c r="G70" s="28" t="s">
+        <v>335</v>
+      </c>
       <c r="H70" s="28" t="s">
-        <v>335</v>
-      </c>
-      <c r="I70" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5886,10 +5876,10 @@
       <c r="D71" s="25" t="s">
         <v>336</v>
       </c>
+      <c r="G71" s="28" t="s">
+        <v>338</v>
+      </c>
       <c r="H71" s="28" t="s">
-        <v>338</v>
-      </c>
-      <c r="I71" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5906,10 +5896,10 @@
       <c r="D72" s="25" t="s">
         <v>341</v>
       </c>
+      <c r="G72" s="28" t="s">
+        <v>342</v>
+      </c>
       <c r="H72" s="28" t="s">
-        <v>342</v>
-      </c>
-      <c r="I72" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -5926,7 +5916,7 @@
       <c r="D73" s="25" t="s">
         <v>345</v>
       </c>
-      <c r="I73" s="28" t="s">
+      <c r="H73" s="28" t="s">
         <v>346</v>
       </c>
     </row>
@@ -5943,7 +5933,7 @@
       <c r="D74" s="25" t="s">
         <v>349</v>
       </c>
-      <c r="I74" s="28" t="s">
+      <c r="H74" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -5960,10 +5950,10 @@
       <c r="D75" s="25" t="s">
         <v>352</v>
       </c>
+      <c r="G75" s="28" t="s">
+        <v>353</v>
+      </c>
       <c r="H75" s="28" t="s">
-        <v>353</v>
-      </c>
-      <c r="I75" s="28" t="s">
         <v>354</v>
       </c>
     </row>
@@ -5980,7 +5970,7 @@
       <c r="D76" s="25" t="s">
         <v>355</v>
       </c>
-      <c r="H76" s="28" t="s">
+      <c r="G76" s="28" t="s">
         <v>357</v>
       </c>
     </row>
@@ -5997,7 +5987,7 @@
       <c r="D77" s="25" t="s">
         <v>358</v>
       </c>
-      <c r="H77" s="28" t="s">
+      <c r="G77" s="28" t="s">
         <v>360</v>
       </c>
     </row>
@@ -6014,7 +6004,7 @@
       <c r="D78" s="25" t="s">
         <v>361</v>
       </c>
-      <c r="H78" s="28" t="s">
+      <c r="G78" s="28" t="s">
         <v>363</v>
       </c>
     </row>
@@ -6031,7 +6021,7 @@
       <c r="D79" s="25" t="s">
         <v>364</v>
       </c>
-      <c r="H79" s="28" t="s">
+      <c r="G79" s="28" t="s">
         <v>366</v>
       </c>
     </row>
@@ -6048,7 +6038,7 @@
       <c r="D80" s="25" t="s">
         <v>369</v>
       </c>
-      <c r="H80" s="28" t="s">
+      <c r="G80" s="28" t="s">
         <v>370</v>
       </c>
     </row>
@@ -6065,10 +6055,10 @@
       <c r="D81" s="25" t="s">
         <v>373</v>
       </c>
+      <c r="G81" s="28" t="s">
+        <v>374</v>
+      </c>
       <c r="H81" s="28" t="s">
-        <v>374</v>
-      </c>
-      <c r="I81" s="28" t="s">
         <v>375</v>
       </c>
     </row>
@@ -6085,7 +6075,7 @@
       <c r="D82" s="25" t="s">
         <v>376</v>
       </c>
-      <c r="H82" s="28" t="s">
+      <c r="G82" s="28" t="s">
         <v>378</v>
       </c>
     </row>
@@ -6102,7 +6092,7 @@
       <c r="D83" s="25" t="s">
         <v>379</v>
       </c>
-      <c r="H83" s="28" t="s">
+      <c r="G83" s="28" t="s">
         <v>381</v>
       </c>
     </row>
@@ -6119,10 +6109,10 @@
       <c r="D84" s="25" t="s">
         <v>384</v>
       </c>
+      <c r="G84" s="28" t="s">
+        <v>385</v>
+      </c>
       <c r="H84" s="28" t="s">
-        <v>385</v>
-      </c>
-      <c r="I84" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -6139,7 +6129,7 @@
       <c r="D85" s="25" t="s">
         <v>387</v>
       </c>
-      <c r="I85" s="28" t="s">
+      <c r="H85" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -6156,10 +6146,10 @@
       <c r="D86" s="25" t="s">
         <v>389</v>
       </c>
+      <c r="G86" s="28" t="s">
+        <v>391</v>
+      </c>
       <c r="H86" s="28" t="s">
-        <v>391</v>
-      </c>
-      <c r="I86" s="28" t="s">
         <v>392</v>
       </c>
     </row>
@@ -6182,7 +6172,7 @@
       <c r="F87" s="32" t="n">
         <v>200</v>
       </c>
-      <c r="H87" s="28" t="s">
+      <c r="G87" s="28" t="s">
         <v>396</v>
       </c>
     </row>
@@ -6205,7 +6195,7 @@
       <c r="F88" s="32" t="n">
         <v>190</v>
       </c>
-      <c r="H88" s="28" t="s">
+      <c r="G88" s="28" t="s">
         <v>400</v>
       </c>
     </row>
@@ -6222,10 +6212,10 @@
       <c r="D89" s="25" t="s">
         <v>403</v>
       </c>
+      <c r="G89" s="28" t="s">
+        <v>404</v>
+      </c>
       <c r="H89" s="28" t="s">
-        <v>404</v>
-      </c>
-      <c r="I89" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6242,10 +6232,10 @@
       <c r="D90" s="25" t="s">
         <v>403</v>
       </c>
+      <c r="G90" s="28" t="s">
+        <v>407</v>
+      </c>
       <c r="H90" s="28" t="s">
-        <v>407</v>
-      </c>
-      <c r="I90" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6262,10 +6252,10 @@
       <c r="D91" s="25" t="s">
         <v>410</v>
       </c>
+      <c r="G91" s="28" t="s">
+        <v>411</v>
+      </c>
       <c r="H91" s="28" t="s">
-        <v>411</v>
-      </c>
-      <c r="I91" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6282,10 +6272,10 @@
       <c r="D92" s="25" t="s">
         <v>414</v>
       </c>
+      <c r="G92" s="28" t="s">
+        <v>415</v>
+      </c>
       <c r="H92" s="28" t="s">
-        <v>415</v>
-      </c>
-      <c r="I92" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6308,7 +6298,7 @@
       <c r="F93" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="H93" s="28" t="s">
+      <c r="G93" s="28" t="s">
         <v>418</v>
       </c>
     </row>
@@ -6331,7 +6321,7 @@
       <c r="F94" s="32" t="s">
         <v>422</v>
       </c>
-      <c r="H94" s="28" t="s">
+      <c r="G94" s="28" t="s">
         <v>423</v>
       </c>
     </row>
@@ -6354,7 +6344,7 @@
       <c r="F95" s="32" t="s">
         <v>428</v>
       </c>
-      <c r="H95" s="28" t="s">
+      <c r="G95" s="28" t="s">
         <v>429</v>
       </c>
     </row>
@@ -6377,7 +6367,7 @@
       <c r="F96" s="32" t="s">
         <v>434</v>
       </c>
-      <c r="H96" s="28" t="s">
+      <c r="G96" s="28" t="s">
         <v>435</v>
       </c>
     </row>
@@ -6394,10 +6384,10 @@
       <c r="D97" s="25" t="s">
         <v>436</v>
       </c>
+      <c r="G97" s="28" t="s">
+        <v>438</v>
+      </c>
       <c r="H97" s="28" t="s">
-        <v>438</v>
-      </c>
-      <c r="I97" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6414,10 +6404,10 @@
       <c r="D98" s="25" t="s">
         <v>439</v>
       </c>
+      <c r="G98" s="28" t="s">
+        <v>441</v>
+      </c>
       <c r="H98" s="28" t="s">
-        <v>441</v>
-      </c>
-      <c r="I98" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6434,10 +6424,10 @@
       <c r="D99" s="25" t="s">
         <v>442</v>
       </c>
+      <c r="G99" s="28" t="s">
+        <v>444</v>
+      </c>
       <c r="H99" s="28" t="s">
-        <v>444</v>
-      </c>
-      <c r="I99" s="28" t="s">
         <v>445</v>
       </c>
     </row>
@@ -6454,10 +6444,10 @@
       <c r="D100" s="25" t="s">
         <v>446</v>
       </c>
+      <c r="G100" s="28" t="s">
+        <v>448</v>
+      </c>
       <c r="H100" s="28" t="s">
-        <v>448</v>
-      </c>
-      <c r="I100" s="28" t="s">
         <v>449</v>
       </c>
     </row>
@@ -6474,10 +6464,10 @@
       <c r="D107" s="25" t="s">
         <v>470</v>
       </c>
+      <c r="G107" s="28" t="s">
+        <v>338</v>
+      </c>
       <c r="H107" s="28" t="s">
-        <v>338</v>
-      </c>
-      <c r="I107" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6494,10 +6484,10 @@
       <c r="D108" s="25" t="s">
         <v>474</v>
       </c>
-      <c r="H108" s="28" t="s">
+      <c r="G108" s="28" t="s">
         <v>338</v>
       </c>
-      <c r="I108" s="28" t="n"/>
+      <c r="H108" s="28" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="25" t="s">
@@ -6512,10 +6502,10 @@
       <c r="D109" s="25" t="s">
         <v>475</v>
       </c>
+      <c r="G109" s="28" t="s">
+        <v>477</v>
+      </c>
       <c r="H109" s="28" t="s">
-        <v>477</v>
-      </c>
-      <c r="I109" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6532,10 +6522,10 @@
       <c r="D110" s="25" t="s">
         <v>478</v>
       </c>
+      <c r="G110" s="28" t="s">
+        <v>477</v>
+      </c>
       <c r="H110" s="28" t="s">
-        <v>477</v>
-      </c>
-      <c r="I110" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6552,10 +6542,10 @@
       <c r="D111" s="25" t="s">
         <v>482</v>
       </c>
-      <c r="H111" s="28" t="s">
+      <c r="G111" s="28" t="s">
         <v>477</v>
       </c>
-      <c r="I111" s="28" t="n"/>
+      <c r="H111" s="28" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="25" t="s">
@@ -6570,10 +6560,10 @@
       <c r="D112" s="25" t="s">
         <v>483</v>
       </c>
+      <c r="G112" s="28" t="s">
+        <v>485</v>
+      </c>
       <c r="H112" s="28" t="s">
-        <v>485</v>
-      </c>
-      <c r="I112" s="28" t="s">
         <v>328</v>
       </c>
     </row>
@@ -6590,10 +6580,10 @@
       <c r="D113" s="25" t="s">
         <v>486</v>
       </c>
+      <c r="G113" s="28" t="s">
+        <v>485</v>
+      </c>
       <c r="H113" s="28" t="s">
-        <v>485</v>
-      </c>
-      <c r="I113" s="28" t="s">
         <v>328</v>
       </c>
     </row>
@@ -6610,10 +6600,10 @@
       <c r="D114" s="25" t="s">
         <v>488</v>
       </c>
+      <c r="G114" s="28" t="s">
+        <v>485</v>
+      </c>
       <c r="H114" s="28" t="s">
-        <v>485</v>
-      </c>
-      <c r="I114" s="28" t="s">
         <v>328</v>
       </c>
     </row>
@@ -6630,10 +6620,10 @@
       <c r="D115" s="25" t="s">
         <v>490</v>
       </c>
+      <c r="G115" s="28" t="s">
+        <v>485</v>
+      </c>
       <c r="H115" s="28" t="s">
-        <v>485</v>
-      </c>
-      <c r="I115" s="28" t="s">
         <v>328</v>
       </c>
     </row>
@@ -6650,10 +6640,10 @@
       <c r="D116" s="25" t="s">
         <v>492</v>
       </c>
+      <c r="G116" s="28" t="s">
+        <v>323</v>
+      </c>
       <c r="H116" s="28" t="s">
-        <v>323</v>
-      </c>
-      <c r="I116" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6670,10 +6660,10 @@
       <c r="D117" s="25" t="s">
         <v>496</v>
       </c>
+      <c r="G117" s="28" t="s">
+        <v>497</v>
+      </c>
       <c r="H117" s="28" t="s">
-        <v>497</v>
-      </c>
-      <c r="I117" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6690,10 +6680,10 @@
       <c r="D118" s="25" t="s">
         <v>498</v>
       </c>
+      <c r="G118" s="28" t="s">
+        <v>500</v>
+      </c>
       <c r="H118" s="28" t="s">
-        <v>500</v>
-      </c>
-      <c r="I118" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6710,10 +6700,10 @@
       <c r="D119" s="25" t="s">
         <v>503</v>
       </c>
+      <c r="G119" s="28" t="s">
+        <v>504</v>
+      </c>
       <c r="H119" s="28" t="s">
-        <v>504</v>
-      </c>
-      <c r="I119" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6730,10 +6720,10 @@
       <c r="D120" s="25" t="s">
         <v>505</v>
       </c>
+      <c r="G120" s="28" t="s">
+        <v>500</v>
+      </c>
       <c r="H120" s="28" t="s">
-        <v>500</v>
-      </c>
-      <c r="I120" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6750,10 +6740,10 @@
       <c r="D121" s="25" t="s">
         <v>432</v>
       </c>
-      <c r="H121" s="28" t="s">
+      <c r="G121" s="28" t="s">
         <v>509</v>
       </c>
-      <c r="I121" s="28" t="n"/>
+      <c r="H121" s="28" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="25" t="s">
@@ -6768,10 +6758,10 @@
       <c r="D122" s="25" t="s">
         <v>512</v>
       </c>
-      <c r="H122" s="28" t="s">
+      <c r="G122" s="28" t="s">
         <v>513</v>
       </c>
-      <c r="I122" s="28" t="n"/>
+      <c r="H122" s="28" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="25" t="s">
@@ -6786,10 +6776,10 @@
       <c r="D123" s="25" t="s">
         <v>516</v>
       </c>
-      <c r="H123" s="28" t="s">
+      <c r="G123" s="28" t="s">
         <v>517</v>
       </c>
-      <c r="I123" s="28" t="n"/>
+      <c r="H123" s="28" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="25" t="s">
@@ -6804,10 +6794,10 @@
       <c r="D124" s="25" t="s">
         <v>520</v>
       </c>
+      <c r="G124" s="28" t="s">
+        <v>521</v>
+      </c>
       <c r="H124" s="28" t="s">
-        <v>521</v>
-      </c>
-      <c r="I124" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -6824,10 +6814,10 @@
       <c r="D125" s="25" t="s">
         <v>524</v>
       </c>
+      <c r="G125" s="28" t="s">
+        <v>521</v>
+      </c>
       <c r="H125" s="28" t="s">
-        <v>521</v>
-      </c>
-      <c r="I125" s="28" t="s">
         <v>525</v>
       </c>
     </row>
@@ -6844,10 +6834,10 @@
       <c r="D126" s="25" t="s">
         <v>528</v>
       </c>
+      <c r="G126" s="28" t="s">
+        <v>521</v>
+      </c>
       <c r="H126" s="28" t="s">
-        <v>521</v>
-      </c>
-      <c r="I126" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -6864,10 +6854,10 @@
       <c r="D127" s="25" t="s">
         <v>529</v>
       </c>
-      <c r="H127" s="28" t="s">
+      <c r="G127" s="28" t="s">
         <v>531</v>
       </c>
-      <c r="I127" s="28" t="n"/>
+      <c r="H127" s="28" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="25" t="s">
@@ -6882,10 +6872,10 @@
       <c r="D128" s="25" t="s">
         <v>534</v>
       </c>
-      <c r="H128" s="28" t="s">
+      <c r="G128" s="28" t="s">
         <v>535</v>
       </c>
-      <c r="I128" s="28" t="n"/>
+      <c r="H128" s="28" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="25" t="s">
@@ -6900,10 +6890,10 @@
       <c r="D129" s="25" t="s">
         <v>538</v>
       </c>
-      <c r="H129" s="28" t="s">
+      <c r="G129" s="28" t="s">
         <v>539</v>
       </c>
-      <c r="I129" s="28" t="n"/>
+      <c r="H129" s="28" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="25" t="s">
@@ -6918,10 +6908,10 @@
       <c r="D130" s="25" t="s">
         <v>542</v>
       </c>
-      <c r="H130" s="28" t="s">
+      <c r="G130" s="28" t="s">
         <v>543</v>
       </c>
-      <c r="I130" s="28" t="n"/>
+      <c r="H130" s="28" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="25" t="s">
@@ -6936,10 +6926,10 @@
       <c r="D131" s="25" t="s">
         <v>546</v>
       </c>
-      <c r="H131" s="28" t="s">
+      <c r="G131" s="28" t="s">
         <v>547</v>
       </c>
-      <c r="I131" s="28" t="n"/>
+      <c r="H131" s="28" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="25" t="s">
@@ -6954,10 +6944,10 @@
       <c r="D132" s="25" t="s">
         <v>550</v>
       </c>
-      <c r="H132" s="28" t="s">
+      <c r="G132" s="28" t="s">
         <v>551</v>
       </c>
-      <c r="I132" s="28" t="n"/>
+      <c r="H132" s="28" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="25" t="s">
@@ -6972,10 +6962,10 @@
       <c r="D133" s="25" t="s">
         <v>554</v>
       </c>
-      <c r="H133" s="28" t="s">
+      <c r="G133" s="28" t="s">
         <v>555</v>
       </c>
-      <c r="I133" s="28" t="n"/>
+      <c r="H133" s="28" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="25" t="s">
@@ -6990,10 +6980,10 @@
       <c r="D134" s="25" t="s">
         <v>559</v>
       </c>
-      <c r="H134" s="28" t="s">
+      <c r="G134" s="28" t="s">
         <v>560</v>
       </c>
-      <c r="I134" s="28" t="n"/>
+      <c r="H134" s="28" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="25" t="s">
@@ -7008,10 +6998,10 @@
       <c r="D135" s="25" t="s">
         <v>561</v>
       </c>
-      <c r="H135" s="28" t="s">
+      <c r="G135" s="28" t="s">
         <v>563</v>
       </c>
-      <c r="I135" s="28" t="n"/>
+      <c r="H135" s="28" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="25" t="s">
@@ -7026,10 +7016,10 @@
       <c r="D136" s="25" t="s">
         <v>564</v>
       </c>
-      <c r="H136" s="28" t="s">
+      <c r="G136" s="28" t="s">
         <v>566</v>
       </c>
-      <c r="I136" s="28" t="n"/>
+      <c r="H136" s="28" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="25" t="s">
@@ -7044,10 +7034,10 @@
       <c r="D137" s="25" t="s">
         <v>567</v>
       </c>
+      <c r="G137" s="28" t="s">
+        <v>569</v>
+      </c>
       <c r="H137" s="28" t="s">
-        <v>569</v>
-      </c>
-      <c r="I137" s="28" t="s">
         <v>570</v>
       </c>
     </row>
@@ -7064,10 +7054,10 @@
       <c r="D138" s="25" t="s">
         <v>571</v>
       </c>
+      <c r="G138" s="28" t="s">
+        <v>569</v>
+      </c>
       <c r="H138" s="28" t="s">
-        <v>569</v>
-      </c>
-      <c r="I138" s="28" t="s">
         <v>573</v>
       </c>
     </row>
@@ -7084,10 +7074,10 @@
       <c r="D139" s="25" t="s">
         <v>576</v>
       </c>
-      <c r="H139" s="28" t="s">
+      <c r="G139" s="28" t="s">
         <v>577</v>
       </c>
-      <c r="I139" s="28" t="n"/>
+      <c r="H139" s="28" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="25" t="s">
@@ -7102,10 +7092,10 @@
       <c r="D140" s="25" t="s">
         <v>580</v>
       </c>
+      <c r="G140" s="28" t="s">
+        <v>581</v>
+      </c>
       <c r="H140" s="28" t="s">
-        <v>581</v>
-      </c>
-      <c r="I140" s="28" t="s">
         <v>582</v>
       </c>
     </row>
@@ -7122,10 +7112,10 @@
       <c r="D141" s="25" t="s">
         <v>585</v>
       </c>
+      <c r="G141" s="28" t="s">
+        <v>586</v>
+      </c>
       <c r="H141" s="28" t="s">
-        <v>586</v>
-      </c>
-      <c r="I141" s="28" t="s">
         <v>582</v>
       </c>
     </row>
@@ -7142,10 +7132,10 @@
       <c r="D142" s="25" t="s">
         <v>589</v>
       </c>
+      <c r="G142" s="28" t="s">
+        <v>590</v>
+      </c>
       <c r="H142" s="28" t="s">
-        <v>590</v>
-      </c>
-      <c r="I142" s="28" t="s">
         <v>582</v>
       </c>
     </row>
@@ -7162,10 +7152,10 @@
       <c r="D143" s="25" t="s">
         <v>593</v>
       </c>
-      <c r="H143" s="28" t="s">
+      <c r="G143" s="28" t="s">
         <v>594</v>
       </c>
-      <c r="I143" s="28" t="n"/>
+      <c r="H143" s="28" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="25" t="s">
@@ -7180,10 +7170,10 @@
       <c r="D144" s="25" t="s">
         <v>597</v>
       </c>
-      <c r="H144" s="28" t="s">
+      <c r="G144" s="28" t="s">
         <v>598</v>
       </c>
-      <c r="I144" s="28" t="n"/>
+      <c r="H144" s="28" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="25" t="s">
@@ -7198,10 +7188,10 @@
       <c r="D145" s="25" t="s">
         <v>601</v>
       </c>
+      <c r="G145" s="28" t="s">
+        <v>602</v>
+      </c>
       <c r="H145" s="28" t="s">
-        <v>602</v>
-      </c>
-      <c r="I145" s="28" t="s">
         <v>603</v>
       </c>
     </row>
@@ -7218,10 +7208,10 @@
       <c r="D146" s="25" t="s">
         <v>604</v>
       </c>
+      <c r="G146" s="28" t="s">
+        <v>606</v>
+      </c>
       <c r="H146" s="28" t="s">
-        <v>606</v>
-      </c>
-      <c r="I146" s="28" t="s">
         <v>274</v>
       </c>
     </row>
@@ -7238,10 +7228,10 @@
       <c r="D147" s="25" t="s">
         <v>607</v>
       </c>
+      <c r="G147" s="28" t="s">
+        <v>609</v>
+      </c>
       <c r="H147" s="28" t="s">
-        <v>609</v>
-      </c>
-      <c r="I147" s="28" t="s">
         <v>314</v>
       </c>
     </row>
@@ -7258,10 +7248,10 @@
       <c r="D148" s="25" t="s">
         <v>612</v>
       </c>
-      <c r="H148" s="28" t="s">
+      <c r="G148" s="28" t="s">
         <v>613</v>
       </c>
-      <c r="I148" s="28" t="n"/>
+      <c r="H148" s="28" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="25" t="s">
@@ -7276,10 +7266,10 @@
       <c r="D149" s="25" t="s">
         <v>616</v>
       </c>
-      <c r="H149" s="28" t="s">
+      <c r="G149" s="28" t="s">
         <v>617</v>
       </c>
-      <c r="I149" s="28" t="n"/>
+      <c r="H149" s="28" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="25" t="s">
@@ -7294,10 +7284,10 @@
       <c r="D150" s="25" t="s">
         <v>618</v>
       </c>
-      <c r="H150" s="28" t="s">
+      <c r="G150" s="28" t="s">
         <v>620</v>
       </c>
-      <c r="I150" s="28" t="n"/>
+      <c r="H150" s="28" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="25" t="s">
@@ -7312,10 +7302,10 @@
       <c r="D151" s="25" t="s">
         <v>621</v>
       </c>
-      <c r="H151" s="28" t="s">
+      <c r="G151" s="28" t="s">
         <v>623</v>
       </c>
-      <c r="I151" s="28" t="n"/>
+      <c r="H151" s="28" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="25" t="s">
@@ -7330,10 +7320,10 @@
       <c r="D152" s="25" t="s">
         <v>911</v>
       </c>
-      <c r="H152" s="28" t="s">
+      <c r="G152" s="28" t="s">
         <v>626</v>
       </c>
-      <c r="I152" s="28" t="n"/>
+      <c r="H152" s="28" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="25" t="s">
@@ -7348,10 +7338,10 @@
       <c r="D153" s="25" t="s">
         <v>627</v>
       </c>
-      <c r="H153" s="28" t="s">
+      <c r="G153" s="28" t="s">
         <v>370</v>
       </c>
-      <c r="I153" s="28" t="n"/>
+      <c r="H153" s="28" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="25" t="s">
@@ -7366,10 +7356,10 @@
       <c r="D154" s="25" t="s">
         <v>894</v>
       </c>
-      <c r="H154" s="28" t="s">
+      <c r="G154" s="28" t="s">
         <v>632</v>
       </c>
-      <c r="I154" s="28" t="n"/>
+      <c r="H154" s="28" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="25" t="s">
@@ -7384,10 +7374,10 @@
       <c r="D155" s="25" t="s">
         <v>917</v>
       </c>
+      <c r="G155" s="28" t="s">
+        <v>635</v>
+      </c>
       <c r="H155" s="28" t="s">
-        <v>635</v>
-      </c>
-      <c r="I155" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7404,10 +7394,10 @@
       <c r="D156" s="25" t="s">
         <v>926</v>
       </c>
+      <c r="G156" s="28" t="s">
+        <v>635</v>
+      </c>
       <c r="H156" s="28" t="s">
-        <v>635</v>
-      </c>
-      <c r="I156" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7424,10 +7414,10 @@
       <c r="D157" s="25" t="s">
         <v>931</v>
       </c>
+      <c r="G157" s="28" t="s">
+        <v>640</v>
+      </c>
       <c r="H157" s="28" t="s">
-        <v>640</v>
-      </c>
-      <c r="I157" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7444,10 +7434,10 @@
       <c r="D158" s="25" t="s">
         <v>641</v>
       </c>
+      <c r="G158" s="28" t="s">
+        <v>643</v>
+      </c>
       <c r="H158" s="28" t="s">
-        <v>643</v>
-      </c>
-      <c r="I158" s="28" t="s">
         <v>644</v>
       </c>
     </row>
@@ -7464,10 +7454,10 @@
       <c r="D159" s="25" t="s">
         <v>645</v>
       </c>
+      <c r="G159" s="28" t="s">
+        <v>643</v>
+      </c>
       <c r="H159" s="28" t="s">
-        <v>643</v>
-      </c>
-      <c r="I159" s="28" t="s">
         <v>644</v>
       </c>
     </row>
@@ -7484,10 +7474,10 @@
       <c r="D160" s="25" t="s">
         <v>647</v>
       </c>
+      <c r="G160" s="28" t="s">
+        <v>643</v>
+      </c>
       <c r="H160" s="28" t="s">
-        <v>643</v>
-      </c>
-      <c r="I160" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7504,10 +7494,10 @@
       <c r="D161" s="25" t="s">
         <v>649</v>
       </c>
+      <c r="G161" s="28" t="s">
+        <v>643</v>
+      </c>
       <c r="H161" s="28" t="s">
-        <v>643</v>
-      </c>
-      <c r="I161" s="28" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7524,10 +7514,10 @@
       <c r="D162" s="25" t="s">
         <v>651</v>
       </c>
+      <c r="G162" s="28" t="s">
+        <v>643</v>
+      </c>
       <c r="H162" s="28" t="s">
-        <v>643</v>
-      </c>
-      <c r="I162" s="28" t="s">
         <v>653</v>
       </c>
     </row>
@@ -7544,10 +7534,10 @@
       <c r="D163" s="25" t="s">
         <v>654</v>
       </c>
+      <c r="G163" s="28" t="s">
+        <v>643</v>
+      </c>
       <c r="H163" s="28" t="s">
-        <v>643</v>
-      </c>
-      <c r="I163" s="28" t="s">
         <v>653</v>
       </c>
     </row>
@@ -7564,10 +7554,10 @@
       <c r="D166" s="25" t="s">
         <v>664</v>
       </c>
-      <c r="H166" s="28" t="s">
+      <c r="G166" s="28" t="s">
         <v>666</v>
       </c>
-      <c r="I166" s="28" t="n"/>
+      <c r="H166" s="28" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="25" t="s">
@@ -7582,10 +7572,10 @@
       <c r="D167" s="25" t="s">
         <v>667</v>
       </c>
-      <c r="H167" s="28" t="s">
+      <c r="G167" s="28" t="s">
         <v>669</v>
       </c>
-      <c r="I167" s="28" t="n"/>
+      <c r="H167" s="28" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="25" t="s">
@@ -7600,7 +7590,7 @@
       <c r="D168" s="25" t="s">
         <v>913</v>
       </c>
-      <c r="H168" t="s">
+      <c r="G168" t="s">
         <v>626</v>
       </c>
     </row>
@@ -7617,7 +7607,7 @@
       <c r="D169" s="25" t="s">
         <v>915</v>
       </c>
-      <c r="H169" t="s">
+      <c r="G169" t="s">
         <v>626</v>
       </c>
     </row>
@@ -7634,10 +7624,10 @@
       <c r="D170" s="25" t="s">
         <v>920</v>
       </c>
+      <c r="G170" t="s">
+        <v>635</v>
+      </c>
       <c r="H170" t="s">
-        <v>635</v>
-      </c>
-      <c r="I170" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7654,10 +7644,10 @@
       <c r="D171" s="25" t="s">
         <v>922</v>
       </c>
+      <c r="G171" t="s">
+        <v>635</v>
+      </c>
       <c r="H171" t="s">
-        <v>635</v>
-      </c>
-      <c r="I171" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7674,10 +7664,10 @@
       <c r="D172" s="25" t="s">
         <v>924</v>
       </c>
+      <c r="G172" t="s">
+        <v>635</v>
+      </c>
       <c r="H172" t="s">
-        <v>635</v>
-      </c>
-      <c r="I172" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7694,10 +7684,10 @@
       <c r="D173" s="25" t="s">
         <v>928</v>
       </c>
+      <c r="G173" t="s">
+        <v>635</v>
+      </c>
       <c r="H173" t="s">
-        <v>635</v>
-      </c>
-      <c r="I173" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7714,10 +7704,10 @@
       <c r="D174" s="25" t="s">
         <v>929</v>
       </c>
+      <c r="G174" t="s">
+        <v>635</v>
+      </c>
       <c r="H174" t="s">
-        <v>635</v>
-      </c>
-      <c r="I174" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7734,10 +7724,10 @@
       <c r="D175" s="25" t="s">
         <v>930</v>
       </c>
+      <c r="G175" t="s">
+        <v>635</v>
+      </c>
       <c r="H175" t="s">
-        <v>635</v>
-      </c>
-      <c r="I175" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7754,10 +7744,10 @@
       <c r="D176" s="25" t="s">
         <v>933</v>
       </c>
+      <c r="G176" t="s">
+        <v>640</v>
+      </c>
       <c r="H176" t="s">
-        <v>640</v>
-      </c>
-      <c r="I176" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7774,10 +7764,10 @@
       <c r="D177" s="25" t="s">
         <v>934</v>
       </c>
+      <c r="G177" t="s">
+        <v>640</v>
+      </c>
       <c r="H177" t="s">
-        <v>640</v>
-      </c>
-      <c r="I177" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7794,10 +7784,10 @@
       <c r="D178" s="25" t="s">
         <v>935</v>
       </c>
+      <c r="G178" t="s">
+        <v>640</v>
+      </c>
       <c r="H178" t="s">
-        <v>640</v>
-      </c>
-      <c r="I178" t="s">
         <v>386</v>
       </c>
     </row>
@@ -7820,7 +7810,7 @@
       <c r="F179" s="32" t="n">
         <v>84.1</v>
       </c>
-      <c r="H179" t="s">
+      <c r="G179" t="s">
         <v>435</v>
       </c>
     </row>
@@ -7843,7 +7833,7 @@
       <c r="F180" s="32" t="n">
         <v>84.1</v>
       </c>
-      <c r="H180" t="s">
+      <c r="G180" t="s">
         <v>435</v>
       </c>
     </row>
@@ -7866,7 +7856,7 @@
       <c r="F181" s="32" t="n">
         <v>84.1</v>
       </c>
-      <c r="H181" t="s">
+      <c r="G181" t="s">
         <v>435</v>
       </c>
     </row>
@@ -7883,7 +7873,7 @@
       <c r="D182" s="25" t="s">
         <v>718</v>
       </c>
-      <c r="H182" t="s">
+      <c r="G182" t="s">
         <v>513</v>
       </c>
     </row>
@@ -7900,7 +7890,7 @@
       <c r="D183" s="25" t="s">
         <v>719</v>
       </c>
-      <c r="H183" t="s">
+      <c r="G183" t="s">
         <v>513</v>
       </c>
     </row>
@@ -7917,7 +7907,7 @@
       <c r="D184" s="25" t="s">
         <v>720</v>
       </c>
-      <c r="H184" t="s">
+      <c r="G184" t="s">
         <v>513</v>
       </c>
     </row>
@@ -7934,7 +7924,7 @@
       <c r="D185" s="25" t="s">
         <v>721</v>
       </c>
-      <c r="H185" t="s">
+      <c r="G185" t="s">
         <v>517</v>
       </c>
     </row>
@@ -7951,7 +7941,7 @@
       <c r="D186" s="25" t="s">
         <v>722</v>
       </c>
-      <c r="H186" t="s">
+      <c r="G186" t="s">
         <v>517</v>
       </c>
     </row>
@@ -7968,7 +7958,7 @@
       <c r="D187" s="25" t="s">
         <v>723</v>
       </c>
-      <c r="H187" t="s">
+      <c r="G187" t="s">
         <v>517</v>
       </c>
     </row>
@@ -7991,7 +7981,7 @@
       <c r="F188" s="32" t="n">
         <v>100</v>
       </c>
-      <c r="H188" t="s">
+      <c r="G188" t="s">
         <v>976</v>
       </c>
     </row>
@@ -8022,7 +8012,7 @@
       <c r="F189" s="32" t="n">
         <v>46</v>
       </c>
-      <c r="H189" t="inlineStr">
+      <c r="G189" t="inlineStr">
         <is>
           <t xml:space="preserve">offset, imprenta offset, tirada grande, papel obra</t>
         </is>

</xml_diff>

<commit_message>
feat(tg-catalogo): completar 'Modo de cálculo' en los 295 tramos que dependían del fallback
La etapa 7 (e6883eb) cargó la columna solo en los 4 materiales nuevos; el
resto del catálogo (176 materiales, 295 tramos) seguía con la celda vacía,
resuelta en silencio por el prefijo de Unidad. Se completa con el MISMO
valor que ya calculaba ese fallback (pliego/unidad/hoja/paquete/pack/metro
lineal/talonario → proporcional, m2 → superficie): ningún precio se mueve,
166/166 casos y validar-catalogo sin errores.

Script nuevo visor/scripts/completar-modo-calculo.mjs (dry-run + --apply,
mismo molde que etapa7-modo-calculo.mjs).

Pendiente, no resuelto acá: chunk.ts (arma lo que ingesta el bot) llama a
modoDe(unidad) sin pasar la columna en sus 5 call sites — solo
build-flow.mjs la lee. Hoy coincide por construcción; si algún valor de la
columna llegara a contradecir el prefijo de Unidad, LLM y auditor
calcularían con modos distintos sin aviso. Cablear eso es tarea aparte.
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v4.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v4.xlsx
@@ -8546,6 +8546,9 @@
       <c r="J2" s="35" t="n">
         <v>0.3</v>
       </c>
+      <c r="O2" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="15">
       <c r="A3" s="26" t="s">
@@ -8563,6 +8566,9 @@
       <c r="E3" s="33" t="n">
         <v>2200</v>
       </c>
+      <c r="O3" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="15">
       <c r="A4" s="26" t="s">
@@ -8580,6 +8586,9 @@
       <c r="E4" s="33" t="n">
         <v>2000</v>
       </c>
+      <c r="O4" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="15">
       <c r="A5" s="26" t="s">
@@ -8597,6 +8606,9 @@
       <c r="E5" s="33" t="n">
         <v>1900</v>
       </c>
+      <c r="O5" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="15">
       <c r="A6" s="26" t="s">
@@ -8612,6 +8624,9 @@
         <v>1710</v>
       </c>
       <c r="G6" s="34" t="n"/>
+      <c r="O6" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="15">
       <c r="A7" s="26" t="s">
@@ -8639,6 +8654,9 @@
       <c r="J7" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O7" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="15">
       <c r="A8" s="26" t="s">
@@ -8654,6 +8672,9 @@
         <v>1620</v>
       </c>
       <c r="G8" s="34" t="n"/>
+      <c r="O8" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="15">
       <c r="A9" s="26" t="s">
@@ -8681,6 +8702,9 @@
       <c r="J9" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O9" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="15">
       <c r="A10" s="26" t="s">
@@ -8699,6 +8723,9 @@
         <v>2160</v>
       </c>
       <c r="G10" s="34" t="n"/>
+      <c r="O10" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="26" t="s">
@@ -8714,6 +8741,9 @@
         <v>1920</v>
       </c>
       <c r="G11" s="34" t="n"/>
+      <c r="O11" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="15">
       <c r="A12" s="26" t="s">
@@ -8741,6 +8771,9 @@
       <c r="J12" s="35" t="n">
         <v>0.3</v>
       </c>
+      <c r="O12" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="15">
       <c r="A13" s="26" t="s">
@@ -8759,6 +8792,9 @@
         <v>2520</v>
       </c>
       <c r="G13" s="34" t="n"/>
+      <c r="O13" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="15">
       <c r="A14" s="26" t="s">
@@ -8774,6 +8810,9 @@
         <v>2240</v>
       </c>
       <c r="G14" s="34" t="n"/>
+      <c r="O14" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="15">
       <c r="A15" s="26" t="s">
@@ -8801,6 +8840,9 @@
       <c r="J15" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O15" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="15">
       <c r="A16" s="26" t="s">
@@ -8819,6 +8861,9 @@
         <v>2340</v>
       </c>
       <c r="G16" s="34" t="n"/>
+      <c r="O16" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="15">
       <c r="A17" s="26" t="s">
@@ -8834,6 +8879,9 @@
         <v>2080</v>
       </c>
       <c r="G17" s="34" t="n"/>
+      <c r="O17" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="15">
       <c r="A18" s="26" t="s">
@@ -8861,6 +8909,9 @@
       <c r="J18" s="35" t="n">
         <v>0.3</v>
       </c>
+      <c r="O18" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="15">
       <c r="A19" s="26" t="s">
@@ -8879,6 +8930,9 @@
         <v>2700</v>
       </c>
       <c r="G19" s="34" t="n"/>
+      <c r="O19" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="15">
       <c r="A20" s="26" t="s">
@@ -8894,6 +8948,9 @@
         <v>2400</v>
       </c>
       <c r="G20" s="34" t="n"/>
+      <c r="O20" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="15">
       <c r="A21" s="26" t="s">
@@ -8912,6 +8969,9 @@
         <v>0.5</v>
       </c>
       <c r="G21" s="34" t="n"/>
+      <c r="O21" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="15">
       <c r="A22" s="26" t="s">
@@ -8930,6 +8990,9 @@
         <v>0.5</v>
       </c>
       <c r="G22" s="34" t="n"/>
+      <c r="O22" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="15">
       <c r="A23" s="26" t="s">
@@ -8948,6 +9011,9 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="34" t="n"/>
+      <c r="O23" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="15">
       <c r="A24" s="26" t="s">
@@ -8966,6 +9032,9 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="34" t="n"/>
+      <c r="O24" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="15">
       <c r="A25" s="26" t="s">
@@ -8984,6 +9053,9 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="34" t="n"/>
+      <c r="O25" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="15">
       <c r="A26" s="26" t="s">
@@ -9001,6 +9073,9 @@
       <c r="L26" s="28" t="s">
         <v>684</v>
       </c>
+      <c r="O26" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="15">
       <c r="A27" s="26" t="s">
@@ -9018,6 +9093,9 @@
       <c r="L27" s="28" t="s">
         <v>685</v>
       </c>
+      <c r="O27" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="15">
       <c r="A28" s="26" t="s">
@@ -9035,6 +9113,9 @@
       <c r="L28" s="28" t="s">
         <v>686</v>
       </c>
+      <c r="O28" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="15">
       <c r="A29" s="26" t="s">
@@ -9052,6 +9133,9 @@
       <c r="L29" s="28" t="s">
         <v>687</v>
       </c>
+      <c r="O29" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="15">
       <c r="A30" s="26" t="s">
@@ -9069,6 +9153,9 @@
       <c r="L30" s="28" t="s">
         <v>688</v>
       </c>
+      <c r="O30" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="15">
       <c r="A31" s="26" t="s">
@@ -9086,6 +9173,9 @@
       <c r="L31" s="28" t="s">
         <v>689</v>
       </c>
+      <c r="O31" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="15">
       <c r="A32" s="26" t="s">
@@ -9103,6 +9193,9 @@
       <c r="L32" s="28" t="s">
         <v>684</v>
       </c>
+      <c r="O32" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="15">
       <c r="A33" s="26" t="s">
@@ -9120,6 +9213,9 @@
       <c r="L33" s="28" t="s">
         <v>685</v>
       </c>
+      <c r="O33" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="15">
       <c r="A34" s="26" t="s">
@@ -9137,6 +9233,9 @@
       <c r="L34" s="28" t="s">
         <v>686</v>
       </c>
+      <c r="O34" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="15">
       <c r="A35" s="26" t="s">
@@ -9154,6 +9253,9 @@
       <c r="L35" s="28" t="s">
         <v>687</v>
       </c>
+      <c r="O35" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="15">
       <c r="A36" s="26" t="s">
@@ -9171,6 +9273,9 @@
       <c r="L36" s="28" t="s">
         <v>684</v>
       </c>
+      <c r="O36" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="15">
       <c r="A37" s="26" t="s">
@@ -9188,6 +9293,9 @@
       <c r="L37" s="28" t="s">
         <v>685</v>
       </c>
+      <c r="O37" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="15">
       <c r="A38" s="26" t="s">
@@ -9205,6 +9313,9 @@
       <c r="L38" s="28" t="s">
         <v>686</v>
       </c>
+      <c r="O38" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="15">
       <c r="A39" s="26" t="s">
@@ -9222,6 +9333,9 @@
       <c r="L39" s="28" t="s">
         <v>687</v>
       </c>
+      <c r="O39" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="15">
       <c r="A40" s="26" t="s">
@@ -9236,6 +9350,9 @@
       <c r="E40" s="33" t="n">
         <v>35000</v>
       </c>
+      <c r="O40" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="15">
       <c r="A41" s="26" t="s">
@@ -9250,6 +9367,9 @@
       <c r="E41" s="33" t="n">
         <v>25000</v>
       </c>
+      <c r="O41" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="15">
       <c r="A42" s="26" t="s">
@@ -9264,6 +9384,9 @@
       <c r="E42" s="33" t="n">
         <v>54000</v>
       </c>
+      <c r="O42" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
       <c r="A43" s="26" t="s">
@@ -9284,6 +9407,9 @@
       <c r="K43" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O43" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="15">
       <c r="A44" s="26" t="s">
@@ -9301,6 +9427,9 @@
       <c r="E44" s="33" t="n">
         <v>220</v>
       </c>
+      <c r="O44" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="15">
       <c r="A45" s="26" t="s">
@@ -9318,6 +9447,9 @@
       <c r="E45" s="33" t="n">
         <v>190</v>
       </c>
+      <c r="O45" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
       <c r="A46" s="26" t="s">
@@ -9332,6 +9464,9 @@
       <c r="E46" s="33" t="n">
         <v>180</v>
       </c>
+      <c r="O46" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">
       <c r="A47" s="26" t="s">
@@ -9352,6 +9487,9 @@
       <c r="K47" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O47" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="15">
       <c r="A48" s="26" t="s">
@@ -9369,6 +9507,9 @@
       <c r="E48" s="33" t="n">
         <v>2500</v>
       </c>
+      <c r="O48" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="15">
       <c r="A49" s="26" t="s">
@@ -9386,6 +9527,9 @@
       <c r="E49" s="33" t="n">
         <v>2300</v>
       </c>
+      <c r="O49" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="15">
       <c r="A50" s="26" t="s">
@@ -9403,6 +9547,9 @@
       <c r="E50" s="33" t="n">
         <v>2100</v>
       </c>
+      <c r="O50" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="15">
       <c r="A51" s="26" t="s">
@@ -9417,6 +9564,9 @@
       <c r="E51" s="33" t="n">
         <v>1900</v>
       </c>
+      <c r="O51" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="15">
       <c r="A52" s="26" t="s">
@@ -9437,6 +9587,9 @@
       <c r="K52" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O52" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="15">
       <c r="A53" s="26" t="s">
@@ -9454,6 +9607,9 @@
       <c r="E53" s="33" t="n">
         <v>2800</v>
       </c>
+      <c r="O53" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="15">
       <c r="A54" s="26" t="s">
@@ -9471,6 +9627,9 @@
       <c r="E54" s="33" t="n">
         <v>2600</v>
       </c>
+      <c r="O54" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="15">
       <c r="A55" s="26" t="s">
@@ -9488,6 +9647,9 @@
       <c r="E55" s="33" t="n">
         <v>2400</v>
       </c>
+      <c r="O55" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="15">
       <c r="A56" s="26" t="s">
@@ -9502,6 +9664,9 @@
       <c r="E56" s="33" t="n">
         <v>2300</v>
       </c>
+      <c r="O56" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="15">
       <c r="A57" s="26" t="s">
@@ -9522,6 +9687,9 @@
       <c r="K57" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O57" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="15">
       <c r="A58" s="26" t="s">
@@ -9539,6 +9707,9 @@
       <c r="E58" s="33" t="n">
         <v>3400</v>
       </c>
+      <c r="O58" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="15">
       <c r="A59" s="26" t="s">
@@ -9556,6 +9727,9 @@
       <c r="E59" s="33" t="n">
         <v>3000</v>
       </c>
+      <c r="O59" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="15">
       <c r="A60" s="26" t="s">
@@ -9570,6 +9744,9 @@
       <c r="E60" s="33" t="n">
         <v>2600</v>
       </c>
+      <c r="O60" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="15">
       <c r="A61" s="26" t="s">
@@ -9590,6 +9767,9 @@
       <c r="K61" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O61" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="15">
       <c r="A62" s="26" t="s">
@@ -9607,6 +9787,9 @@
       <c r="E62" s="33" t="n">
         <v>3800</v>
       </c>
+      <c r="O62" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="15">
       <c r="A63" s="26" t="s">
@@ -9624,6 +9807,9 @@
       <c r="E63" s="33" t="n">
         <v>3200</v>
       </c>
+      <c r="O63" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="15">
       <c r="A64" s="26" t="s">
@@ -9638,6 +9824,9 @@
       <c r="E64" s="33" t="n">
         <v>2800</v>
       </c>
+      <c r="O64" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="15">
       <c r="A65" s="26" t="s">
@@ -9658,6 +9847,9 @@
       <c r="K65" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O65" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="15">
       <c r="A66" s="26" t="s">
@@ -9675,6 +9867,9 @@
       <c r="E66" s="33" t="n">
         <v>150</v>
       </c>
+      <c r="O66" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="15">
       <c r="A67" s="26" t="s">
@@ -9692,6 +9887,9 @@
       <c r="E67" s="33" t="n">
         <v>80</v>
       </c>
+      <c r="O67" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="15">
       <c r="A68" s="26" t="s">
@@ -9706,6 +9904,9 @@
       <c r="E68" s="33" t="n">
         <v>70</v>
       </c>
+      <c r="O68" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" s="26" t="s">
@@ -9726,6 +9927,9 @@
       <c r="K69" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O69" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="15">
       <c r="A70" s="26" t="s">
@@ -9743,6 +9947,9 @@
       <c r="E70" s="33" t="n">
         <v>200</v>
       </c>
+      <c r="O70" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="15">
       <c r="A71" s="26" t="s">
@@ -9760,6 +9967,9 @@
       <c r="E71" s="33" t="n">
         <v>120</v>
       </c>
+      <c r="O71" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="26" t="s">
@@ -9774,6 +9984,9 @@
       <c r="E72" s="33" t="n">
         <v>110</v>
       </c>
+      <c r="O72" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="15">
       <c r="A73" s="26" t="s">
@@ -9794,6 +10007,9 @@
       <c r="K73" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O73" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="15">
       <c r="A74" s="26" t="s">
@@ -9808,6 +10024,9 @@
       <c r="E74" s="33" t="n">
         <v>70</v>
       </c>
+      <c r="O74" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="15">
       <c r="A75" s="26" t="s">
@@ -9828,6 +10047,9 @@
       <c r="K75" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O75" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="15">
       <c r="A76" s="26" t="s">
@@ -9845,6 +10067,9 @@
       <c r="E76" s="33" t="n">
         <v>96</v>
       </c>
+      <c r="O76" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="15">
       <c r="A77" s="26" t="s">
@@ -9862,6 +10087,9 @@
       <c r="E77" s="33" t="n">
         <v>88</v>
       </c>
+      <c r="O77" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="15">
       <c r="A78" s="26" t="s">
@@ -9879,6 +10107,9 @@
       <c r="E78" s="33" t="n">
         <v>86</v>
       </c>
+      <c r="O78" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="15">
       <c r="A79" s="26" t="s">
@@ -9893,6 +10124,9 @@
       <c r="E79" s="33" t="n">
         <v>84</v>
       </c>
+      <c r="O79" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="15">
       <c r="A80" s="26" t="s">
@@ -9910,6 +10144,9 @@
       <c r="K80" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O80" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="15">
       <c r="A81" s="26" t="s">
@@ -9927,6 +10164,9 @@
       <c r="K81" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O81" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="15">
       <c r="A82" s="26" t="s">
@@ -9944,6 +10184,9 @@
       <c r="K82" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O82" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="15">
       <c r="A83" s="26" t="s">
@@ -9961,6 +10204,9 @@
       <c r="K83" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O83" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="15">
       <c r="A84" s="26" t="s">
@@ -9981,6 +10227,9 @@
       <c r="L84" s="28" t="s">
         <v>697</v>
       </c>
+      <c r="O84" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="15">
       <c r="A85" s="26" t="s">
@@ -10001,6 +10250,9 @@
       <c r="L85" s="28" t="s">
         <v>698</v>
       </c>
+      <c r="O85" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="15">
       <c r="A86" s="26" t="s">
@@ -10018,6 +10270,9 @@
       <c r="K86" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O86" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="15">
       <c r="A87" s="26" t="s">
@@ -10035,6 +10290,9 @@
       <c r="E87" s="33" t="n">
         <v>7000</v>
       </c>
+      <c r="O87" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="15">
       <c r="A88" s="26" t="s">
@@ -10052,6 +10310,9 @@
       <c r="E88" s="33" t="n">
         <v>5000</v>
       </c>
+      <c r="O88" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="15">
       <c r="A89" s="26" t="s">
@@ -10072,6 +10333,9 @@
       <c r="L89" s="28" t="s">
         <v>699</v>
       </c>
+      <c r="O89" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="15">
       <c r="A90" s="26" t="s">
@@ -10092,6 +10356,9 @@
       <c r="L90" s="28" t="s">
         <v>700</v>
       </c>
+      <c r="O90" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="15">
       <c r="A91" s="26" t="s">
@@ -10112,6 +10379,9 @@
       <c r="L91" s="28" t="s">
         <v>700</v>
       </c>
+      <c r="O91" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="15">
       <c r="A92" s="26" t="s">
@@ -10132,6 +10402,9 @@
       <c r="L92" s="28" t="s">
         <v>700</v>
       </c>
+      <c r="O92" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="15">
       <c r="A93" s="26" t="s">
@@ -10152,6 +10425,9 @@
       <c r="L93" s="28" t="s">
         <v>700</v>
       </c>
+      <c r="O93" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="15">
       <c r="A94" s="26" t="s">
@@ -10172,6 +10448,9 @@
       <c r="L94" s="28" t="s">
         <v>700</v>
       </c>
+      <c r="O94" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="15">
       <c r="A95" s="26" t="s">
@@ -10192,6 +10471,9 @@
       <c r="K95" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O95" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="15">
       <c r="A96" s="26" t="s">
@@ -10209,6 +10491,9 @@
       <c r="K96" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O96" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="15">
       <c r="A97" s="26" t="s">
@@ -10223,6 +10508,9 @@
       <c r="E97" s="33" t="n">
         <v>5000</v>
       </c>
+      <c r="O97" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="15">
       <c r="A98" s="26" t="s">
@@ -10237,6 +10525,9 @@
       <c r="E98" s="33" t="n">
         <v>4000</v>
       </c>
+      <c r="O98" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="15">
       <c r="A99" s="26" t="s">
@@ -10251,6 +10542,9 @@
       <c r="E99" s="33" t="n">
         <v>12000</v>
       </c>
+      <c r="O99" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="15">
       <c r="A100" s="26" t="s">
@@ -10265,6 +10559,9 @@
       <c r="E100" s="33" t="n">
         <v>30000</v>
       </c>
+      <c r="O100" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="15">
       <c r="A101" s="26" t="s">
@@ -10279,6 +10576,9 @@
       <c r="E101" s="33" t="n">
         <v>99000</v>
       </c>
+      <c r="O101" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="15">
       <c r="A102" s="26" t="s">
@@ -10299,6 +10599,9 @@
       <c r="K102" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O102" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="15">
       <c r="A103" s="26" t="s">
@@ -10316,6 +10619,9 @@
       <c r="E103" s="33" t="n">
         <v>3400</v>
       </c>
+      <c r="O103" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="15">
       <c r="A104" s="26" t="s">
@@ -10333,6 +10639,9 @@
       <c r="E104" s="33" t="n">
         <v>3000</v>
       </c>
+      <c r="O104" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="15">
       <c r="A105" s="26" t="s">
@@ -10347,6 +10656,9 @@
       <c r="E105" s="33" t="n">
         <v>2600</v>
       </c>
+      <c r="O105" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="15">
       <c r="A106" s="26" t="s">
@@ -10367,6 +10679,9 @@
       <c r="K106" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O106" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="15">
       <c r="A107" s="26" t="s">
@@ -10384,6 +10699,9 @@
       <c r="E107" s="33" t="n">
         <v>3800</v>
       </c>
+      <c r="O107" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="15">
       <c r="A108" s="26" t="s">
@@ -10401,6 +10719,9 @@
       <c r="E108" s="33" t="n">
         <v>3200</v>
       </c>
+      <c r="O108" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="15">
       <c r="A109" s="26" t="s">
@@ -10415,6 +10736,9 @@
       <c r="E109" s="33" t="n">
         <v>2800</v>
       </c>
+      <c r="O109" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="15">
       <c r="A110" s="26" t="s">
@@ -10432,6 +10756,9 @@
       <c r="K110" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O110" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="15">
       <c r="A111" s="26" t="s">
@@ -10446,6 +10773,9 @@
       <c r="E111" s="33" t="n">
         <v>38000</v>
       </c>
+      <c r="O111" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="15">
       <c r="A112" s="26" t="s">
@@ -10460,6 +10790,9 @@
       <c r="E112" s="33" t="n">
         <v>32000</v>
       </c>
+      <c r="O112" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="15">
       <c r="A113" s="26" t="s">
@@ -10474,6 +10807,9 @@
       <c r="E113" s="33" t="n">
         <v>10500</v>
       </c>
+      <c r="O113" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="15">
       <c r="A114" s="26" t="s">
@@ -10491,6 +10827,9 @@
       <c r="K114" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O114" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="15">
       <c r="A115" s="26" t="s">
@@ -10505,6 +10844,9 @@
       <c r="E115" s="33" t="n">
         <v>4800</v>
       </c>
+      <c r="O115" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="15">
       <c r="A116" s="26" t="s">
@@ -10525,6 +10867,9 @@
       <c r="L116" t="s">
         <v>980</v>
       </c>
+      <c r="O116" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="15">
       <c r="A117" s="26" t="s">
@@ -10542,6 +10887,9 @@
       <c r="F117" s="28" t="s">
         <v>706</v>
       </c>
+      <c r="O117" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="15">
       <c r="A118" s="26" t="s">
@@ -10562,6 +10910,9 @@
       <c r="L118" t="s">
         <v>978</v>
       </c>
+      <c r="O118" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="15">
       <c r="A119" s="26" t="s">
@@ -10576,6 +10927,9 @@
       <c r="E119" s="33" t="n">
         <v>8000</v>
       </c>
+      <c r="O119" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="15">
       <c r="A120" s="26" t="s">
@@ -10593,6 +10947,9 @@
       <c r="E120" s="33" t="n">
         <v>1900</v>
       </c>
+      <c r="O120" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="15">
       <c r="A121" s="26" t="s">
@@ -10610,6 +10967,9 @@
       <c r="E121" s="33" t="n">
         <v>1400</v>
       </c>
+      <c r="O121" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="15">
       <c r="A122" s="26" t="s">
@@ -10624,6 +10984,9 @@
       <c r="E122" s="33" t="n">
         <v>1000</v>
       </c>
+      <c r="O122" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="15">
       <c r="A123" s="26" t="s">
@@ -10638,6 +11001,9 @@
       <c r="E123" s="33" t="n">
         <v>61360</v>
       </c>
+      <c r="O123" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="15">
       <c r="A124" s="26" t="s">
@@ -10652,6 +11018,9 @@
       <c r="E124" s="33" t="n">
         <v>65200</v>
       </c>
+      <c r="O124" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="26" t="s">
@@ -10679,6 +11048,9 @@
       <c r="J125" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O125" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="26" t="s">
@@ -10696,6 +11068,9 @@
       <c r="E126" s="33" t="n">
         <v>1080</v>
       </c>
+      <c r="O126" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="26" t="s">
@@ -10713,6 +11088,9 @@
       <c r="E127" s="33" t="n">
         <v>1020</v>
       </c>
+      <c r="O127" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="26" t="s">
@@ -10730,6 +11108,9 @@
       <c r="E128" s="33" t="n">
         <v>960</v>
       </c>
+      <c r="O128" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="26" t="s">
@@ -10747,6 +11128,9 @@
       <c r="E129" s="33" t="n">
         <v>900</v>
       </c>
+      <c r="O129" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="26" t="s">
@@ -10764,6 +11148,9 @@
       <c r="E130" s="33" t="n">
         <v>840</v>
       </c>
+      <c r="O130" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="26" t="s">
@@ -10791,6 +11178,9 @@
       <c r="J131" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O131" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="26" t="s">
@@ -10808,6 +11198,9 @@
       <c r="E132" s="33" t="n">
         <v>1440</v>
       </c>
+      <c r="O132" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="26" t="s">
@@ -10825,6 +11218,9 @@
       <c r="E133" s="33" t="n">
         <v>1360</v>
       </c>
+      <c r="O133" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="26" t="s">
@@ -10842,6 +11238,9 @@
       <c r="E134" s="33" t="n">
         <v>1280</v>
       </c>
+      <c r="O134" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="26" t="s">
@@ -10859,6 +11258,9 @@
       <c r="E135" s="33" t="n">
         <v>1200</v>
       </c>
+      <c r="O135" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="26" t="s">
@@ -10876,6 +11278,9 @@
       <c r="E136" s="33" t="n">
         <v>1120</v>
       </c>
+      <c r="O136" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="26" t="s">
@@ -10903,6 +11308,9 @@
       <c r="J137" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O137" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="26" t="s">
@@ -10920,6 +11328,9 @@
       <c r="E138" s="33" t="n">
         <v>1530</v>
       </c>
+      <c r="O138" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="26" t="s">
@@ -10937,6 +11348,9 @@
       <c r="E139" s="33" t="n">
         <v>1445</v>
       </c>
+      <c r="O139" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="26" t="s">
@@ -10954,6 +11368,9 @@
       <c r="E140" s="33" t="n">
         <v>1360</v>
       </c>
+      <c r="O140" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="26" t="s">
@@ -10971,6 +11388,9 @@
       <c r="E141" s="33" t="n">
         <v>1275</v>
       </c>
+      <c r="O141" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="26" t="s">
@@ -10988,6 +11408,9 @@
       <c r="E142" s="33" t="n">
         <v>1190</v>
       </c>
+      <c r="O142" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="26" t="s">
@@ -11015,6 +11438,9 @@
       <c r="J143" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O143" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="26" t="s">
@@ -11032,6 +11458,9 @@
       <c r="E144" s="33" t="n">
         <v>1620</v>
       </c>
+      <c r="O144" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="26" t="s">
@@ -11049,6 +11478,9 @@
       <c r="E145" s="33" t="n">
         <v>1530</v>
       </c>
+      <c r="O145" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="26" t="s">
@@ -11066,6 +11498,9 @@
       <c r="E146" s="33" t="n">
         <v>1440</v>
       </c>
+      <c r="O146" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="26" t="s">
@@ -11083,6 +11518,9 @@
       <c r="E147" s="33" t="n">
         <v>1350</v>
       </c>
+      <c r="O147" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="26" t="s">
@@ -11100,6 +11538,9 @@
       <c r="E148" s="33" t="n">
         <v>1260</v>
       </c>
+      <c r="O148" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="26" t="s">
@@ -11127,6 +11568,9 @@
       <c r="J149" s="35" t="n">
         <v>0</v>
       </c>
+      <c r="O149" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="26" t="s">
@@ -11144,6 +11588,9 @@
       <c r="E150" s="33" t="n">
         <v>1620</v>
       </c>
+      <c r="O150" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="26" t="s">
@@ -11161,6 +11608,9 @@
       <c r="E151" s="33" t="n">
         <v>1530</v>
       </c>
+      <c r="O151" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="26" t="s">
@@ -11178,6 +11628,9 @@
       <c r="E152" s="33" t="n">
         <v>1440</v>
       </c>
+      <c r="O152" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="26" t="s">
@@ -11195,6 +11648,9 @@
       <c r="E153" s="33" t="n">
         <v>1350</v>
       </c>
+      <c r="O153" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="26" t="s">
@@ -11212,6 +11668,9 @@
       <c r="E154" s="33" t="n">
         <v>1260</v>
       </c>
+      <c r="O154" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="26" t="s">
@@ -11232,6 +11691,9 @@
       <c r="L160" s="28" t="s">
         <v>699</v>
       </c>
+      <c r="O160" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="26" t="s">
@@ -11252,6 +11714,9 @@
       <c r="L161" s="28" t="s">
         <v>699</v>
       </c>
+      <c r="O161" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="26" t="s">
@@ -11272,6 +11737,9 @@
       <c r="L162" s="28" t="s">
         <v>713</v>
       </c>
+      <c r="O162" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="26" t="s">
@@ -11292,6 +11760,9 @@
       <c r="L163" s="28" t="s">
         <v>713</v>
       </c>
+      <c r="O163" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="26" t="s">
@@ -11312,6 +11783,9 @@
       <c r="L164" s="28" t="s">
         <v>713</v>
       </c>
+      <c r="O164" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="26" t="s">
@@ -11332,6 +11806,9 @@
       <c r="L165" s="28" t="s">
         <v>698</v>
       </c>
+      <c r="O165" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="26" t="s">
@@ -11352,6 +11829,9 @@
       <c r="L166" s="28" t="s">
         <v>698</v>
       </c>
+      <c r="O166" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="26" t="s">
@@ -11372,6 +11852,9 @@
       <c r="L167" s="28" t="s">
         <v>698</v>
       </c>
+      <c r="O167" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="26" t="s">
@@ -11392,6 +11875,9 @@
       <c r="L168" s="28" t="s">
         <v>698</v>
       </c>
+      <c r="O168" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="26" t="s">
@@ -11412,6 +11898,9 @@
       <c r="L169" s="28" t="s">
         <v>697</v>
       </c>
+      <c r="O169" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="26" t="s">
@@ -11433,6 +11922,9 @@
         <v>714</v>
       </c>
       <c r="K170" s="28" t="n"/>
+      <c r="O170" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="26" t="s">
@@ -11453,6 +11945,9 @@
       <c r="K171" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O171" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="26" t="s">
@@ -11471,6 +11966,9 @@
         <v>230</v>
       </c>
       <c r="K172" s="28" t="n"/>
+      <c r="O172" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="26" t="s">
@@ -11489,6 +11987,9 @@
         <v>160</v>
       </c>
       <c r="K173" s="28" t="n"/>
+      <c r="O173" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="26" t="s">
@@ -11504,6 +12005,9 @@
         <v>150</v>
       </c>
       <c r="K174" s="28" t="n"/>
+      <c r="O174" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="26" t="s">
@@ -11524,6 +12028,9 @@
       <c r="K175" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O175" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="26" t="s">
@@ -11542,6 +12049,9 @@
         <v>280</v>
       </c>
       <c r="K176" s="28" t="n"/>
+      <c r="O176" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="26" t="s">
@@ -11560,6 +12070,9 @@
         <v>200</v>
       </c>
       <c r="K177" s="28" t="n"/>
+      <c r="O177" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="26" t="s">
@@ -11578,6 +12091,9 @@
         <v>190</v>
       </c>
       <c r="K178" s="28" t="n"/>
+      <c r="O178" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="26" t="s">
@@ -11593,6 +12109,9 @@
         <v>170</v>
       </c>
       <c r="K179" s="28" t="n"/>
+      <c r="O179" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="26" t="s">
@@ -11613,6 +12132,9 @@
       <c r="K180" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O180" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="26" t="s">
@@ -11628,6 +12150,9 @@
         <v>150</v>
       </c>
       <c r="K181" s="28" t="n"/>
+      <c r="O181" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="26" t="s">
@@ -11648,6 +12173,9 @@
       <c r="K182" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O182" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="26" t="s">
@@ -11667,6 +12195,9 @@
       </c>
       <c r="G183" s="28" t="n"/>
       <c r="K183" s="28" t="n"/>
+      <c r="O183" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="26" t="s">
@@ -11685,6 +12216,9 @@
         <v>170</v>
       </c>
       <c r="K184" s="28" t="n"/>
+      <c r="O184" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="26" t="s">
@@ -11703,6 +12237,9 @@
         <v>166</v>
       </c>
       <c r="K185" s="28" t="n"/>
+      <c r="O185" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="26" t="s">
@@ -11718,6 +12255,9 @@
         <v>164</v>
       </c>
       <c r="K186" s="28" t="n"/>
+      <c r="O186" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="26" t="s">
@@ -11738,6 +12278,9 @@
       <c r="L187" t="s">
         <v>978</v>
       </c>
+      <c r="O187" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="26" t="s">
@@ -11758,6 +12301,9 @@
       <c r="L188" t="s">
         <v>978</v>
       </c>
+      <c r="O188" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="26" t="s">
@@ -11778,6 +12324,9 @@
       <c r="L189" t="s">
         <v>978</v>
       </c>
+      <c r="O189" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="26" t="s">
@@ -11798,6 +12347,9 @@
       <c r="L190" t="s">
         <v>510</v>
       </c>
+      <c r="O190" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="26" t="s">
@@ -11818,6 +12370,9 @@
       <c r="L191" t="s">
         <v>510</v>
       </c>
+      <c r="O191" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="26" t="s">
@@ -11838,6 +12393,9 @@
       <c r="L192" t="s">
         <v>510</v>
       </c>
+      <c r="O192" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="26" t="s">
@@ -11858,6 +12416,9 @@
       <c r="L193" t="s">
         <v>510</v>
       </c>
+      <c r="O193" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="26" t="s">
@@ -11878,6 +12439,9 @@
       <c r="L194" t="s">
         <v>979</v>
       </c>
+      <c r="O194" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="26" t="s">
@@ -11898,6 +12462,9 @@
       <c r="L195" t="s">
         <v>979</v>
       </c>
+      <c r="O195" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="26" t="s">
@@ -11918,6 +12485,9 @@
       <c r="L196" t="s">
         <v>979</v>
       </c>
+      <c r="O196" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="26" t="s">
@@ -11938,6 +12508,9 @@
       <c r="L197" t="s">
         <v>979</v>
       </c>
+      <c r="O197" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="26" t="s">
@@ -11956,6 +12529,9 @@
       <c r="K198" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O198" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="26" t="s">
@@ -11974,6 +12550,9 @@
       <c r="K199" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O199" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="26" t="s">
@@ -11992,6 +12571,9 @@
       <c r="K200" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O200" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="26" t="s">
@@ -12012,6 +12594,9 @@
       <c r="G201" s="28" t="s">
         <v>724</v>
       </c>
+      <c r="O201" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="26" t="s">
@@ -12032,6 +12617,9 @@
       <c r="G202" s="28" t="s">
         <v>725</v>
       </c>
+      <c r="O202" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="26" t="s">
@@ -12052,6 +12640,9 @@
       <c r="G203" s="28" t="s">
         <v>726</v>
       </c>
+      <c r="O203" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="26" t="s">
@@ -12069,6 +12660,9 @@
       <c r="F204" s="28" t="n">
         <v>0.5</v>
       </c>
+      <c r="O204" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="26" t="s">
@@ -12086,6 +12680,9 @@
       <c r="F205" s="28" t="n">
         <v>0.5</v>
       </c>
+      <c r="O205" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="26" t="s">
@@ -12103,6 +12700,9 @@
       <c r="F206" s="28" t="n">
         <v>0.5</v>
       </c>
+      <c r="O206" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="26" t="s">
@@ -12123,6 +12723,9 @@
       <c r="G207" s="28" t="s">
         <v>727</v>
       </c>
+      <c r="O207" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="26" t="s">
@@ -12146,6 +12749,9 @@
       <c r="L208" t="s">
         <v>980</v>
       </c>
+      <c r="O208" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="26" t="s">
@@ -12167,6 +12773,9 @@
       <c r="K209" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O209" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="26" t="s">
@@ -12185,6 +12794,9 @@
         <v>7800</v>
       </c>
       <c r="F210" s="28" t="n"/>
+      <c r="O210" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="26" t="s">
@@ -12206,6 +12818,9 @@
       <c r="G211" s="28" t="s">
         <v>714</v>
       </c>
+      <c r="O211" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="26" t="s">
@@ -12223,6 +12838,9 @@
       <c r="F212" s="28" t="n">
         <v>0.5</v>
       </c>
+      <c r="O212" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="26" t="s">
@@ -12240,6 +12858,9 @@
       <c r="F213" s="28" t="n">
         <v>0.5</v>
       </c>
+      <c r="O213" t="s">
+        <v>1111</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="26" t="s">
@@ -12258,6 +12879,9 @@
       <c r="K214" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O214" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="26" t="s">
@@ -12276,6 +12900,9 @@
       <c r="K215" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O215" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="26" t="s">
@@ -12294,6 +12921,9 @@
       <c r="K216" s="28" t="s">
         <v>144</v>
       </c>
+      <c r="O216" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="26" t="s">
@@ -12314,6 +12944,9 @@
       <c r="L217" s="28" t="s">
         <v>730</v>
       </c>
+      <c r="O217" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="26" t="s">
@@ -12334,6 +12967,9 @@
       <c r="L218" s="28" t="s">
         <v>730</v>
       </c>
+      <c r="O218" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="26" t="s">
@@ -12354,6 +12990,9 @@
       <c r="L219" s="28" t="s">
         <v>732</v>
       </c>
+      <c r="O219" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="26" t="s">
@@ -12374,6 +13013,9 @@
       <c r="L220" s="28" t="s">
         <v>732</v>
       </c>
+      <c r="O220" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="26" t="s">
@@ -12394,6 +13036,9 @@
       <c r="L221" s="28" t="s">
         <v>734</v>
       </c>
+      <c r="O221" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="26" t="s">
@@ -12414,6 +13059,9 @@
       <c r="L222" s="28" t="s">
         <v>734</v>
       </c>
+      <c r="O222" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="26" t="s">
@@ -12434,6 +13082,9 @@
       <c r="L223" s="28" t="s">
         <v>591</v>
       </c>
+      <c r="O223" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="26" t="s">
@@ -12454,6 +13105,9 @@
       <c r="L224" s="28" t="s">
         <v>591</v>
       </c>
+      <c r="O224" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="26" t="s">
@@ -12474,6 +13128,9 @@
       <c r="L225" s="28" t="s">
         <v>591</v>
       </c>
+      <c r="O225" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="26" t="s">
@@ -12494,6 +13151,9 @@
       <c r="L226" s="28" t="s">
         <v>591</v>
       </c>
+      <c r="O226" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="26" t="s">
@@ -12514,6 +13174,9 @@
       <c r="L227" s="28" t="s">
         <v>591</v>
       </c>
+      <c r="O227" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="26" t="s">
@@ -12534,6 +13197,9 @@
       <c r="L228" s="28" t="s">
         <v>595</v>
       </c>
+      <c r="O228" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="26" t="s">
@@ -12554,6 +13220,9 @@
       <c r="L229" s="28" t="s">
         <v>595</v>
       </c>
+      <c r="O229" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="26" t="s">
@@ -12574,6 +13243,9 @@
       <c r="L230" s="28" t="s">
         <v>595</v>
       </c>
+      <c r="O230" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="26" t="s">
@@ -12594,6 +13266,9 @@
       <c r="L231" s="28" t="s">
         <v>595</v>
       </c>
+      <c r="O231" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="26" t="s">
@@ -12614,6 +13289,9 @@
       <c r="L232" s="28" t="s">
         <v>595</v>
       </c>
+      <c r="O232" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="26" t="s">
@@ -12632,6 +13310,9 @@
         <v>144</v>
       </c>
       <c r="L233" s="28" t="n"/>
+      <c r="O233" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="26" t="s">
@@ -12650,6 +13331,9 @@
         <v>144</v>
       </c>
       <c r="L234" s="28" t="n"/>
+      <c r="O234" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="26" t="s">
@@ -12668,6 +13352,9 @@
         <v>144</v>
       </c>
       <c r="L235" s="28" t="n"/>
+      <c r="O235" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="26" t="s">
@@ -12686,6 +13373,9 @@
         <v>144</v>
       </c>
       <c r="L236" s="28" t="n"/>
+      <c r="O236" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="26" t="s">
@@ -12706,6 +13396,9 @@
       <c r="L237" s="28" t="s">
         <v>614</v>
       </c>
+      <c r="O237" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="26" t="s">
@@ -12726,6 +13419,9 @@
       <c r="L238" s="28" t="s">
         <v>614</v>
       </c>
+      <c r="O238" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="26" t="s">
@@ -12746,6 +13442,9 @@
       <c r="L239" s="28" t="s">
         <v>614</v>
       </c>
+      <c r="O239" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="26" t="s">
@@ -12766,6 +13465,9 @@
       <c r="L240" s="28" t="s">
         <v>614</v>
       </c>
+      <c r="O240" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="26" t="s">
@@ -12786,6 +13488,9 @@
       <c r="L241" s="28" t="s">
         <v>614</v>
       </c>
+      <c r="O241" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="26" t="s">
@@ -12804,6 +13509,9 @@
         <v>144</v>
       </c>
       <c r="L242" s="28" t="n"/>
+      <c r="O242" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="26" t="s">
@@ -12825,6 +13533,9 @@
         <v>144</v>
       </c>
       <c r="L243" s="28" t="n"/>
+      <c r="O243" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="26" t="s">
@@ -12844,6 +13555,9 @@
       </c>
       <c r="K244" s="28" t="n"/>
       <c r="L244" s="28" t="n"/>
+      <c r="O244" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="26" t="s">
@@ -12866,6 +13580,9 @@
       </c>
       <c r="K245" s="28" t="n"/>
       <c r="L245" s="28" t="n"/>
+      <c r="O245" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="26" t="s">
@@ -12884,6 +13601,9 @@
         <v>144</v>
       </c>
       <c r="L249" s="28" t="n"/>
+      <c r="O249" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="26" t="s">
@@ -12902,6 +13622,9 @@
         <v>144</v>
       </c>
       <c r="L250" s="28" t="n"/>
+      <c r="O250" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="26" t="s">
@@ -12923,6 +13646,9 @@
         <v>144</v>
       </c>
       <c r="L263" s="28" t="n"/>
+      <c r="O263" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="26" t="s">
@@ -12942,6 +13668,9 @@
       </c>
       <c r="K264" s="28" t="n"/>
       <c r="L264" s="28" t="n"/>
+      <c r="O264" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="26" t="s">
@@ -12961,6 +13690,9 @@
       </c>
       <c r="K265" s="28" t="n"/>
       <c r="L265" s="28" t="n"/>
+      <c r="O265" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="26" t="s">
@@ -12983,6 +13715,9 @@
       </c>
       <c r="K266" s="28" t="n"/>
       <c r="L266" s="28" t="n"/>
+      <c r="O266" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="26" t="s">
@@ -13004,6 +13739,9 @@
         <v>144</v>
       </c>
       <c r="L267" s="28" t="n"/>
+      <c r="O267" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="26" t="s">
@@ -13023,6 +13761,9 @@
       </c>
       <c r="K268" s="28" t="n"/>
       <c r="L268" s="28" t="n"/>
+      <c r="O268" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="26" t="s">
@@ -13042,6 +13783,9 @@
       </c>
       <c r="K269" s="28" t="n"/>
       <c r="L269" s="28" t="n"/>
+      <c r="O269" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="26" t="s">
@@ -13064,6 +13808,9 @@
       </c>
       <c r="K270" s="28" t="n"/>
       <c r="L270" s="28" t="n"/>
+      <c r="O270" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="26" t="s">
@@ -13085,6 +13832,9 @@
         <v>144</v>
       </c>
       <c r="L271" s="28" t="n"/>
+      <c r="O271" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="26" t="s">
@@ -13104,6 +13854,9 @@
       </c>
       <c r="K272" s="28" t="n"/>
       <c r="L272" s="28" t="n"/>
+      <c r="O272" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="26" t="s">
@@ -13123,6 +13876,9 @@
       </c>
       <c r="K273" s="28" t="n"/>
       <c r="L273" s="28" t="n"/>
+      <c r="O273" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="26" t="s">
@@ -13145,6 +13901,9 @@
       </c>
       <c r="K274" s="28" t="n"/>
       <c r="L274" s="28" t="n"/>
+      <c r="O274" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="26" t="s">
@@ -13166,6 +13925,9 @@
         <v>144</v>
       </c>
       <c r="L275" s="28" t="n"/>
+      <c r="O275" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="26" t="s">
@@ -13185,6 +13947,9 @@
       </c>
       <c r="K276" s="28" t="n"/>
       <c r="L276" s="28" t="n"/>
+      <c r="O276" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="26" t="s">
@@ -13204,6 +13969,9 @@
       </c>
       <c r="K277" s="28" t="n"/>
       <c r="L277" s="28" t="n"/>
+      <c r="O277" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="26" t="s">
@@ -13226,6 +13994,9 @@
       </c>
       <c r="K278" s="28" t="n"/>
       <c r="L278" s="28" t="n"/>
+      <c r="O278" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="26" t="s">
@@ -13247,6 +14018,9 @@
         <v>144</v>
       </c>
       <c r="L279" s="28" t="n"/>
+      <c r="O279" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="26" t="s">
@@ -13266,6 +14040,9 @@
       </c>
       <c r="K280" s="28" t="n"/>
       <c r="L280" s="28" t="n"/>
+      <c r="O280" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="26" t="s">
@@ -13285,6 +14062,9 @@
       </c>
       <c r="K281" s="28" t="n"/>
       <c r="L281" s="28" t="n"/>
+      <c r="O281" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="26" t="s">
@@ -13307,6 +14087,9 @@
       </c>
       <c r="K282" s="28" t="n"/>
       <c r="L282" s="28" t="n"/>
+      <c r="O282" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="26" t="s">
@@ -13328,6 +14111,9 @@
         <v>144</v>
       </c>
       <c r="L283" s="28" t="n"/>
+      <c r="O283" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="26" t="s">
@@ -13347,6 +14133,9 @@
       </c>
       <c r="K284" s="28" t="n"/>
       <c r="L284" s="28" t="n"/>
+      <c r="O284" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="26" t="s">
@@ -13366,6 +14155,9 @@
       </c>
       <c r="K285" s="28" t="n"/>
       <c r="L285" s="28" t="n"/>
+      <c r="O285" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="26" t="s">
@@ -13388,6 +14180,9 @@
       </c>
       <c r="K286" s="28" t="n"/>
       <c r="L286" s="28" t="n"/>
+      <c r="O286" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="26" t="s">
@@ -13406,6 +14201,9 @@
         <v>144</v>
       </c>
       <c r="L299" s="28" t="n"/>
+      <c r="O299" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="26" t="s">
@@ -13424,6 +14222,9 @@
         <v>144</v>
       </c>
       <c r="L300" s="28" t="n"/>
+      <c r="O300" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="26" t="s">
@@ -13441,6 +14242,9 @@
       <c r="L301" t="s">
         <v>624</v>
       </c>
+      <c r="O301" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="26" t="s">
@@ -13458,6 +14262,9 @@
       <c r="L302" t="s">
         <v>624</v>
       </c>
+      <c r="O302" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="26" t="s">
@@ -13475,6 +14282,9 @@
       <c r="L303" t="s">
         <v>624</v>
       </c>
+      <c r="O303" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="26" t="s">
@@ -13492,6 +14302,9 @@
       <c r="L304" t="s">
         <v>919</v>
       </c>
+      <c r="O304" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="26" t="s">
@@ -13509,6 +14322,9 @@
       <c r="L305" t="s">
         <v>919</v>
       </c>
+      <c r="O305" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="26" t="s">
@@ -13526,6 +14342,9 @@
       <c r="L306" t="s">
         <v>919</v>
       </c>
+      <c r="O306" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="26" t="s">
@@ -13543,6 +14362,9 @@
       <c r="L307" t="s">
         <v>919</v>
       </c>
+      <c r="O307" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="26" t="s">
@@ -13560,6 +14382,9 @@
       <c r="L308" t="s">
         <v>927</v>
       </c>
+      <c r="O308" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="26" t="s">
@@ -13577,6 +14402,9 @@
       <c r="L309" t="s">
         <v>927</v>
       </c>
+      <c r="O309" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="26" t="s">
@@ -13594,6 +14422,9 @@
       <c r="L310" t="s">
         <v>927</v>
       </c>
+      <c r="O310" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="26" t="s">
@@ -13611,6 +14442,9 @@
       <c r="L311" t="s">
         <v>927</v>
       </c>
+      <c r="O311" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="26" t="s">
@@ -13628,6 +14462,9 @@
       <c r="L312" t="s">
         <v>932</v>
       </c>
+      <c r="O312" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="26" t="s">
@@ -13645,6 +14482,9 @@
       <c r="L313" t="s">
         <v>932</v>
       </c>
+      <c r="O313" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="26" t="s">
@@ -13662,6 +14502,9 @@
       <c r="L314" t="s">
         <v>932</v>
       </c>
+      <c r="O314" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="26" t="s">
@@ -13679,6 +14522,9 @@
       <c r="L315" t="s">
         <v>932</v>
       </c>
+      <c r="O315" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="26" t="s">
@@ -13739,6 +14585,9 @@
       <c r="E318" s="33">
         <v>1000</v>
       </c>
+      <c r="O318" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="26" t="s">
@@ -13756,6 +14605,9 @@
       <c r="E319" s="33">
         <v>800</v>
       </c>
+      <c r="O319" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="26" t="s">
@@ -13770,6 +14622,9 @@
       <c r="E320" s="33">
         <v>600</v>
       </c>
+      <c r="O320" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="26" t="s">
@@ -13819,6 +14674,9 @@
       <c r="N322" t="s">
         <v>144</v>
       </c>
+      <c r="O322" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="26" t="s">
@@ -13842,6 +14700,9 @@
       <c r="N323" t="s">
         <v>144</v>
       </c>
+      <c r="O323" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="26" t="s">
@@ -13865,6 +14726,9 @@
       <c r="N324" t="s">
         <v>144</v>
       </c>
+      <c r="O324" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="26" t="s">
@@ -13888,6 +14752,9 @@
       <c r="N325" t="s">
         <v>144</v>
       </c>
+      <c r="O325" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="26" t="s">
@@ -13908,6 +14775,9 @@
       <c r="N326" t="s">
         <v>144</v>
       </c>
+      <c r="O326" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="26" t="s">
@@ -13957,6 +14827,9 @@
       <c r="N328" t="s">
         <v>144</v>
       </c>
+      <c r="O328" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="26" t="s">
@@ -13980,6 +14853,9 @@
       <c r="N329" t="s">
         <v>144</v>
       </c>
+      <c r="O329" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="26" t="s">
@@ -14003,6 +14879,9 @@
       <c r="N330" t="s">
         <v>144</v>
       </c>
+      <c r="O330" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="26" t="s">
@@ -14026,6 +14905,9 @@
       <c r="N331" t="s">
         <v>144</v>
       </c>
+      <c r="O331" t="s">
+        <v>1108</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="26" t="s">
@@ -14045,6 +14927,9 @@
       </c>
       <c r="N332" t="s">
         <v>144</v>
+      </c>
+      <c r="O332" t="s">
+        <v>1108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(tg-catalogo): completar 'Piezas por paquete' donde el número ya vivía en la Unidad
Mismo argumento que la etapa 7 con 'Modo de cálculo': la columna es el
estándar para dejar de depender de texto libre en Unidad, así que se
completa donde corresponde en vez de quedar 'opcional porque el fallback
alcanza'.

36 filas completadas (tarjetas, folletos, perforados, puntas redondeadas,
volantes, hojas membretadas, sobres, talonarios, corte) con el mismo
número que ya extraía paqueteDe() del texto ("paquete de 500 tarjetas" →
500) — no-op de precio, verificado con 166/166 casos y validar-catalogo
sin errores nuevos.

Quedan afuera A PROPÓSITO 2 filas "pack" a secas (fila 101 "Pack 4 libros
de medicina", fila 216 "Promoción cartelería... 6 carteles"): cargarles el
número SÍ cambia el precio real (hoy cotizan como 1 unidad, pasarían a
paquete cerrado de 4 y 6) — decisión pendiente aparte, no mezclada con
este completado que no debía mover nada.
</commit_message>
<xml_diff>
--- a/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v4.xlsx
+++ b/project-context/TerminalGrafica/whatsapp-rag/Catalogo-TG-v4.xlsx
@@ -9076,6 +9076,9 @@
       <c r="O26" t="s">
         <v>1108</v>
       </c>
+      <c r="M26" s="28">
+        <v>100</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="15">
       <c r="A27" s="26" t="s">
@@ -9096,6 +9099,9 @@
       <c r="O27" t="s">
         <v>1108</v>
       </c>
+      <c r="M27" s="28">
+        <v>100</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="15">
       <c r="A28" s="26" t="s">
@@ -9116,6 +9122,9 @@
       <c r="O28" t="s">
         <v>1108</v>
       </c>
+      <c r="M28" s="28">
+        <v>100</v>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="15">
       <c r="A29" s="26" t="s">
@@ -9136,6 +9145,9 @@
       <c r="O29" t="s">
         <v>1108</v>
       </c>
+      <c r="M29" s="28">
+        <v>100</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="15">
       <c r="A30" s="26" t="s">
@@ -9156,6 +9168,9 @@
       <c r="O30" t="s">
         <v>1108</v>
       </c>
+      <c r="M30" s="28">
+        <v>100</v>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="15">
       <c r="A31" s="26" t="s">
@@ -9176,6 +9191,9 @@
       <c r="O31" t="s">
         <v>1108</v>
       </c>
+      <c r="M31" s="28">
+        <v>100</v>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="15">
       <c r="A32" s="26" t="s">
@@ -9196,6 +9214,9 @@
       <c r="O32" t="s">
         <v>1108</v>
       </c>
+      <c r="M32" s="28">
+        <v>500</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="15">
       <c r="A33" s="26" t="s">
@@ -9216,6 +9237,9 @@
       <c r="O33" t="s">
         <v>1108</v>
       </c>
+      <c r="M33" s="28">
+        <v>500</v>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="15">
       <c r="A34" s="26" t="s">
@@ -9236,6 +9260,9 @@
       <c r="O34" t="s">
         <v>1108</v>
       </c>
+      <c r="M34" s="28">
+        <v>500</v>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="15">
       <c r="A35" s="26" t="s">
@@ -9256,6 +9283,9 @@
       <c r="O35" t="s">
         <v>1108</v>
       </c>
+      <c r="M35" s="28">
+        <v>500</v>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="15">
       <c r="A36" s="26" t="s">
@@ -9276,6 +9306,9 @@
       <c r="O36" t="s">
         <v>1108</v>
       </c>
+      <c r="M36" s="28">
+        <v>1000</v>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="15">
       <c r="A37" s="26" t="s">
@@ -9296,6 +9329,9 @@
       <c r="O37" t="s">
         <v>1108</v>
       </c>
+      <c r="M37" s="28">
+        <v>1000</v>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="15">
       <c r="A38" s="26" t="s">
@@ -9316,6 +9352,9 @@
       <c r="O38" t="s">
         <v>1108</v>
       </c>
+      <c r="M38" s="28">
+        <v>1000</v>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="15">
       <c r="A39" s="26" t="s">
@@ -9336,6 +9375,9 @@
       <c r="O39" t="s">
         <v>1108</v>
       </c>
+      <c r="M39" s="28">
+        <v>1000</v>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="15">
       <c r="A40" s="26" t="s">
@@ -9353,6 +9395,9 @@
       <c r="O40" t="s">
         <v>1108</v>
       </c>
+      <c r="M40">
+        <v>500</v>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="15">
       <c r="A41" s="26" t="s">
@@ -9370,6 +9415,9 @@
       <c r="O41" t="s">
         <v>1108</v>
       </c>
+      <c r="M41">
+        <v>100</v>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="15">
       <c r="A42" s="26" t="s">
@@ -9387,6 +9435,9 @@
       <c r="O42" t="s">
         <v>1108</v>
       </c>
+      <c r="M42">
+        <v>10</v>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
       <c r="A43" s="26" t="s">
@@ -10528,6 +10579,9 @@
       <c r="O98" t="s">
         <v>1108</v>
       </c>
+      <c r="M98">
+        <v>500</v>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="15">
       <c r="A99" s="26" t="s">
@@ -10545,6 +10599,9 @@
       <c r="O99" t="s">
         <v>1108</v>
       </c>
+      <c r="M99">
+        <v>500</v>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="15">
       <c r="A100" s="26" t="s">
@@ -13604,6 +13661,9 @@
       <c r="O249" t="s">
         <v>1108</v>
       </c>
+      <c r="M249" s="28">
+        <v>1000</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="26" t="s">
@@ -13625,6 +13685,9 @@
       <c r="O250" t="s">
         <v>1108</v>
       </c>
+      <c r="M250" s="28">
+        <v>1000</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="26" t="s">
@@ -14245,6 +14308,9 @@
       <c r="O301" t="s">
         <v>1108</v>
       </c>
+      <c r="M301">
+        <v>100</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="26" t="s">
@@ -14265,6 +14331,9 @@
       <c r="O302" t="s">
         <v>1108</v>
       </c>
+      <c r="M302">
+        <v>500</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="26" t="s">
@@ -14285,6 +14354,9 @@
       <c r="O303" t="s">
         <v>1108</v>
       </c>
+      <c r="M303">
+        <v>1000</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="26" t="s">
@@ -14305,6 +14377,9 @@
       <c r="O304" t="s">
         <v>1108</v>
       </c>
+      <c r="M304">
+        <v>500</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="26" t="s">
@@ -14325,6 +14400,9 @@
       <c r="O305" t="s">
         <v>1108</v>
       </c>
+      <c r="M305">
+        <v>1000</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="26" t="s">
@@ -14345,6 +14423,9 @@
       <c r="O306" t="s">
         <v>1108</v>
       </c>
+      <c r="M306">
+        <v>2000</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="26" t="s">
@@ -14365,6 +14446,9 @@
       <c r="O307" t="s">
         <v>1108</v>
       </c>
+      <c r="M307">
+        <v>3000</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="26" t="s">
@@ -14385,6 +14469,9 @@
       <c r="O308" t="s">
         <v>1108</v>
       </c>
+      <c r="M308">
+        <v>500</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="26" t="s">
@@ -14405,6 +14492,9 @@
       <c r="O309" t="s">
         <v>1108</v>
       </c>
+      <c r="M309">
+        <v>1000</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="26" t="s">
@@ -14425,6 +14515,9 @@
       <c r="O310" t="s">
         <v>1108</v>
       </c>
+      <c r="M310">
+        <v>2000</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="26" t="s">
@@ -14445,6 +14538,9 @@
       <c r="O311" t="s">
         <v>1108</v>
       </c>
+      <c r="M311">
+        <v>3000</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="26" t="s">
@@ -14465,6 +14561,9 @@
       <c r="O312" t="s">
         <v>1108</v>
       </c>
+      <c r="M312">
+        <v>500</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="26" t="s">
@@ -14485,6 +14584,9 @@
       <c r="O313" t="s">
         <v>1108</v>
       </c>
+      <c r="M313">
+        <v>1000</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="26" t="s">
@@ -14505,6 +14607,9 @@
       <c r="O314" t="s">
         <v>1108</v>
       </c>
+      <c r="M314">
+        <v>2000</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="26" t="s">
@@ -14524,6 +14629,9 @@
       </c>
       <c r="O315" t="s">
         <v>1108</v>
+      </c>
+      <c r="M315">
+        <v>3000</v>
       </c>
     </row>
     <row r="316">

</xml_diff>